<commit_message>
Update Company_Tracker: Saudi Aramco 221 jobs (2026-03-07)
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -945,11 +945,11 @@
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D25" s="24" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Company_Tracker: ADNOC 63 jobs (2026-03-07)
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -531,11 +531,11 @@
         </is>
       </c>
       <c r="C2" s="19" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add CNOOC International (3 jobs, Calgary, Canada) — 4,960 jobs, 30 companies
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -630,431 +630,449 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="15">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>CNOOC International</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="15">
+      <c r="A9" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Dragon Oil</t>
         </is>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="20" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="15">
-      <c r="A9" s="21" t="n">
+    <row r="10" ht="15" customHeight="1" s="15">
+      <c r="A10" s="21" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>ENOC</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="22" t="inlineStr">
-        <is>
-          <t>ENOC</t>
-        </is>
-      </c>
-      <c r="C9" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="15">
-      <c r="A10" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="15">
+      <c r="A11" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>ExxonMobil</t>
         </is>
       </c>
-      <c r="C10" s="19" t="n">
+      <c r="C11" s="19" t="n">
         <v>542</v>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="15">
-      <c r="A11" s="21" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="22" t="inlineStr">
+    <row r="12" ht="15" customHeight="1" s="15">
+      <c r="A12" s="21" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>Halliburton</t>
         </is>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C12" s="23" t="n">
         <v>523</v>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="15">
-      <c r="A12" s="17" t="n">
+    <row r="13" ht="15" customHeight="1" s="15">
+      <c r="A13" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>INOC</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="15">
+      <c r="A14" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>INPEX</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>72</v>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="15">
+      <c r="A15" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>KNPC</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="15">
+      <c r="A16" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>KPC</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="15">
+      <c r="A17" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>Mubadala Energy</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="15">
+      <c r="A18" s="21" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>NIOC</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="15">
+      <c r="A19" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>North Oil Company</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="15">
+      <c r="A20" s="21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>OQ Group</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="15">
+      <c r="A21" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>PDO</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="15">
+      <c r="A22" s="21" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Petrofac</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="15">
+      <c r="A23" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Petronas</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="15">
+      <c r="A24" s="21" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>QatarEnergy</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>284</v>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1" s="15">
+      <c r="A25" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>QatarEnergy LNG</t>
+        </is>
+      </c>
+      <c r="C25" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>INOC</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="15">
-      <c r="A13" s="21" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="22" t="inlineStr">
-        <is>
-          <t>INPEX</t>
-        </is>
-      </c>
-      <c r="C13" s="23" t="n">
-        <v>72</v>
-      </c>
-      <c r="D13" s="24" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="15">
+      <c r="A26" s="21" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>Saudi Aramco</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="n">
+        <v>221</v>
+      </c>
+      <c r="D26" s="24" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="15">
-      <c r="A14" s="17" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>KNPC</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="15">
-      <c r="A15" s="21" t="n">
+    <row r="27" ht="15" customHeight="1" s="15">
+      <c r="A27" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="n">
+        <v>181</v>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="15">
+      <c r="A28" s="21" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="n">
+        <v>824</v>
+      </c>
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="15">
+      <c r="A29" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="n">
+        <v>27</v>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="15">
+      <c r="A30" s="21" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>TotalEnergies</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="n">
+        <v>658</v>
+      </c>
+      <c r="D30" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="15">
+      <c r="A31" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>Woodside Energy</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="22" t="inlineStr">
-        <is>
-          <t>KPC</t>
-        </is>
-      </c>
-      <c r="C15" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="D15" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="15">
-      <c r="A16" s="17" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Mubadala Energy</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="D16" s="20" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1" s="15">
-      <c r="A17" s="21" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="22" t="inlineStr">
-        <is>
-          <t>NIOC</t>
-        </is>
-      </c>
-      <c r="C17" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="15">
-      <c r="A18" s="17" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>North Oil Company</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="15">
-      <c r="A19" s="21" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="22" t="inlineStr">
-        <is>
-          <t>OQ Group</t>
-        </is>
-      </c>
-      <c r="C19" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="D19" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="15">
-      <c r="A20" s="17" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>PDO</t>
-        </is>
-      </c>
-      <c r="C20" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="D20" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="15">
-      <c r="A21" s="21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="22" t="inlineStr">
-        <is>
-          <t>Petrofac</t>
-        </is>
-      </c>
-      <c r="C21" s="23" t="n">
-        <v>55</v>
-      </c>
-      <c r="D21" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="15">
-      <c r="A22" s="17" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Petronas</t>
-        </is>
-      </c>
-      <c r="C22" s="19" t="n">
-        <v>30</v>
-      </c>
-      <c r="D22" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="15">
-      <c r="A23" s="21" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="22" t="inlineStr">
-        <is>
-          <t>QatarEnergy</t>
-        </is>
-      </c>
-      <c r="C23" s="23" t="n">
-        <v>284</v>
-      </c>
-      <c r="D23" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="15">
-      <c r="A24" s="17" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>QatarEnergy LNG</t>
-        </is>
-      </c>
-      <c r="C24" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="D24" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="15">
-      <c r="A25" s="21" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="22" t="inlineStr">
-        <is>
-          <t>Saudi Aramco</t>
-        </is>
-      </c>
-      <c r="C25" s="23" t="n">
-        <v>221</v>
-      </c>
-      <c r="D25" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="15">
-      <c r="A26" s="17" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>Shell</t>
-        </is>
-      </c>
-      <c r="C26" s="19" t="n">
-        <v>181</v>
-      </c>
-      <c r="D26" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="15">
-      <c r="A27" s="21" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="22" t="inlineStr">
-        <is>
-          <t>SLB</t>
-        </is>
-      </c>
-      <c r="C27" s="23" t="n">
-        <v>824</v>
-      </c>
-      <c r="D27" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="15">
-      <c r="A28" s="17" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Suncor</t>
-        </is>
-      </c>
-      <c r="C28" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D28" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="15">
-      <c r="A29" s="21" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="22" t="inlineStr">
-        <is>
-          <t>TotalEnergies</t>
-        </is>
-      </c>
-      <c r="C29" s="23" t="n">
-        <v>658</v>
-      </c>
-      <c r="D29" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="15">
-      <c r="A30" s="17" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="18" t="inlineStr">
-        <is>
-          <t>Woodside Energy</t>
-        </is>
-      </c>
-      <c r="C30" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="D30" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="15">
-      <c r="A31" s="25" t="n"/>
-      <c r="B31" s="26" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="25" t="n"/>
+      <c r="B32" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C31" s="27">
-        <f>SUM(C2:C30)</f>
+      <c r="C32" s="27">
+        <f>SUM(C2:C31)</f>
         <v/>
       </c>
-      <c r="D31" s="25" t="n"/>
+      <c r="D32" s="25" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Scrape PDO from PetroJobs.om — 8 jobs (was 6 placeholder), add SCRAPING_GUIDE entry #20
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -873,11 +873,11 @@
         </is>
       </c>
       <c r="C21" s="19" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D21" s="20" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scrape QatarEnergy LNG from Taleo site — 12 jobs (was 11), add SCRAPING_GUIDE entry #21
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -945,11 +945,11 @@
         </is>
       </c>
       <c r="C25" s="19" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D25" s="20" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scrape Dragon Oil from SAP SuccessFactors — 8 jobs (was 3 placeholder), add SCRAPING_GUIDE entry #23
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -657,11 +657,11 @@
         </is>
       </c>
       <c r="C9" s="19" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add McDermott: 357 jobs from Oracle HCM Cloud (31 companies, 5325 jobs, 126 countries)
- Scraped via Oracle HCM REST API with pagination (25/page, 15 pages)
- Jobs span 18+ countries (UAE 78, Malaysia 65, India 55, Indonesia 41, US 36, UK 19, etc.)
- Categories inferred from job titles (no department field in API)
- Updated SCRAPING_GUIDE.md entry #24 and Company_Tracker.xlsx
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -810,269 +810,282 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="15">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="17" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>McDermott</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="15">
+      <c r="A19" s="21" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>NIOC</t>
         </is>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C19" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="D18" s="24" t="inlineStr">
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="15">
-      <c r="A19" s="17" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
+    <row r="20" ht="15" customHeight="1" s="15">
+      <c r="A20" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>North Oil Company</t>
         </is>
       </c>
-      <c r="C19" s="19" t="n">
+      <c r="C20" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="15">
-      <c r="A20" s="21" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="22" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="15">
+      <c r="A21" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>OQ Group</t>
         </is>
       </c>
-      <c r="C20" s="23" t="n">
+      <c r="C21" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="D20" s="24" t="inlineStr">
+      <c r="D21" s="24" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="15">
-      <c r="A21" s="17" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="15">
+      <c r="A22" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>PDO</t>
         </is>
       </c>
-      <c r="C21" s="19" t="n">
+      <c r="C22" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="D21" s="20" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="15">
-      <c r="A22" s="21" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="22" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="15">
+      <c r="A23" s="21" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>Petrofac</t>
         </is>
       </c>
-      <c r="C22" s="23" t="n">
+      <c r="C23" s="23" t="n">
         <v>55</v>
       </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="D23" s="24" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="15">
-      <c r="A23" s="17" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="15">
+      <c r="A24" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>Petronas</t>
         </is>
       </c>
-      <c r="C23" s="19" t="n">
+      <c r="C24" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="D23" s="20" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="15">
-      <c r="A24" s="21" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="22" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="15">
+      <c r="A25" s="21" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
         <is>
           <t>QatarEnergy</t>
         </is>
       </c>
-      <c r="C24" s="23" t="n">
+      <c r="C25" s="23" t="n">
         <v>284</v>
       </c>
-      <c r="D24" s="24" t="inlineStr">
+      <c r="D25" s="24" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="15">
-      <c r="A25" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="15">
+      <c r="A26" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>QatarEnergy LNG</t>
         </is>
       </c>
-      <c r="C25" s="19" t="n">
+      <c r="C26" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="D25" s="20" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="15">
-      <c r="A26" s="21" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="22" t="inlineStr">
+    <row r="27" ht="15" customHeight="1" s="15">
+      <c r="A27" s="21" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
         <is>
           <t>Saudi Aramco</t>
         </is>
       </c>
-      <c r="C26" s="23" t="n">
+      <c r="C27" s="23" t="n">
         <v>221</v>
       </c>
-      <c r="D26" s="24" t="inlineStr">
+      <c r="D27" s="24" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="15">
-      <c r="A27" s="17" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
+    <row r="28" ht="15" customHeight="1" s="15">
+      <c r="A28" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>Shell</t>
         </is>
       </c>
-      <c r="C27" s="19" t="n">
+      <c r="C28" s="19" t="n">
         <v>181</v>
       </c>
-      <c r="D27" s="20" t="inlineStr">
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="15">
-      <c r="A28" s="21" t="n">
+    <row r="29" ht="15" customHeight="1" s="15">
+      <c r="A29" s="21" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="n">
+        <v>824</v>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="15">
+      <c r="A30" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="22" t="inlineStr">
-        <is>
-          <t>SLB</t>
-        </is>
-      </c>
-      <c r="C28" s="23" t="n">
-        <v>824</v>
-      </c>
-      <c r="D28" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="15">
-      <c r="A29" s="17" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="18" t="inlineStr">
-        <is>
-          <t>Suncor</t>
-        </is>
-      </c>
-      <c r="C29" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D29" s="20" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1" s="15">
-      <c r="A30" s="21" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="22" t="inlineStr">
+    <row r="31" ht="15" customHeight="1" s="15">
+      <c r="A31" s="21" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
         <is>
           <t>TotalEnergies</t>
         </is>
       </c>
-      <c r="C30" s="23" t="n">
+      <c r="C31" s="23" t="n">
         <v>658</v>
       </c>
-      <c r="D30" s="24" t="inlineStr">
+      <c r="D31" s="24" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="15">
-      <c r="A31" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="18" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="18" t="inlineStr">
         <is>
           <t>Woodside Energy</t>
         </is>
       </c>
-      <c r="C31" s="19" t="n">
+      <c r="C32" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="25" t="n"/>
-      <c r="B32" s="26" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="25" t="n"/>
+      <c r="B33" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C32" s="27">
-        <f>SUM(C2:C31)</f>
+      <c r="C33" s="27">
+        <f>SUM(C2:C32)</f>
         <v/>
       </c>
-      <c r="D32" s="25" t="n"/>
+      <c r="D33" s="25" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Add Saipem: 195 jobs from jobs.saipem.com (32 companies, 5520 jobs, 129 countries)
- Scraped via static JSON (positions_saipem.json) from NCorePlat platform
- 17 subsidiaries across 15+ countries (Italy 50, France 32, Offshore 25, Qatar 13, etc.)
- Updated SCRAPING_GUIDE.md entry #25 and Company_Tracker.xlsx
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -967,125 +967,138 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="15">
-      <c r="A27" s="21" t="n">
+      <c r="A27" s="17" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="22" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Saipem</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="15">
+      <c r="A28" s="21" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
         <is>
           <t>Saudi Aramco</t>
         </is>
       </c>
-      <c r="C27" s="23" t="n">
+      <c r="C28" s="23" t="n">
         <v>221</v>
       </c>
-      <c r="D27" s="24" t="inlineStr">
+      <c r="D28" s="24" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="15">
-      <c r="A28" s="17" t="n">
+    <row r="29" ht="15" customHeight="1" s="15">
+      <c r="A29" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="n">
+        <v>181</v>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="15">
+      <c r="A30" s="21" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="n">
+        <v>824</v>
+      </c>
+      <c r="D30" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="15">
+      <c r="A31" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="18" t="inlineStr">
-        <is>
-          <t>Shell</t>
-        </is>
-      </c>
-      <c r="C28" s="19" t="n">
-        <v>181</v>
-      </c>
-      <c r="D28" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="15">
-      <c r="A29" s="21" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="22" t="inlineStr">
-        <is>
-          <t>SLB</t>
-        </is>
-      </c>
-      <c r="C29" s="23" t="n">
-        <v>824</v>
-      </c>
-      <c r="D29" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="15">
-      <c r="A30" s="17" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="18" t="inlineStr">
-        <is>
-          <t>Suncor</t>
-        </is>
-      </c>
-      <c r="C30" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D30" s="20" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="15">
-      <c r="A31" s="21" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="22" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="21" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
         <is>
           <t>TotalEnergies</t>
         </is>
       </c>
-      <c r="C31" s="23" t="n">
+      <c r="C32" s="23" t="n">
         <v>658</v>
       </c>
-      <c r="D31" s="24" t="inlineStr">
+      <c r="D32" s="24" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="17" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="18" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>Woodside Energy</t>
         </is>
       </c>
-      <c r="C32" s="19" t="n">
+      <c r="C33" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="D32" s="20" t="inlineStr">
+      <c r="D33" s="20" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="25" t="n"/>
-      <c r="B33" s="26" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="25" t="n"/>
+      <c r="B34" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C33" s="27">
-        <f>SUM(C2:C32)</f>
+      <c r="C34" s="27">
+        <f>SUM(C2:C33)</f>
         <v/>
       </c>
-      <c r="D33" s="25" t="n"/>
+      <c r="D34" s="25" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Add Technip Energies: 172 jobs from Oracle HCM Cloud (33 companies, 5692 jobs, 129 countries)
- Scraped via Oracle HCM REST API with pagination (25/page, 7 pages)
- Jobs across 15 countries (France 58, UK 27, India 20, Malaysia 15, UAE 11, USA 10, etc.)
- Updated SCRAPING_GUIDE.md entry #26 and Company_Tracker.xlsx
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -1052,53 +1052,66 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="21" t="n">
+      <c r="A32" s="17" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="22" t="inlineStr">
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>Technip Energies</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
         <is>
           <t>TotalEnergies</t>
         </is>
       </c>
-      <c r="C32" s="23" t="n">
+      <c r="C33" s="23" t="n">
         <v>658</v>
       </c>
-      <c r="D32" s="24" t="inlineStr">
+      <c r="D33" s="24" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="17" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="18" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="18" t="inlineStr">
         <is>
           <t>Woodside Energy</t>
         </is>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C34" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="D33" s="20" t="inlineStr">
+      <c r="D34" s="20" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="25" t="n"/>
-      <c r="B34" s="26" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="25" t="n"/>
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C34" s="27">
-        <f>SUM(C2:C33)</f>
+      <c r="C35" s="27">
+        <f>SUM(C2:C34)</f>
         <v/>
       </c>
-      <c r="D34" s="25" t="n"/>
+      <c r="D35" s="25" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Add NMDC: 52 jobs from Oracle HCM Cloud (34 companies, 5744 jobs, 129 countries)
- Scraped via Oracle HCM REST API (all jobs in 3 pages)
- All 52 jobs in UAE (Abu Dhabi) — marine, dredging, construction focus
- Updated SCRAPING_GUIDE.md entry #27 and Company_Tracker.xlsx
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -841,128 +841,123 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="15">
-      <c r="A20" s="17" t="n">
+      <c r="A20" s="21" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>NMDC</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="15">
+      <c r="A21" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>North Oil Company</t>
         </is>
       </c>
-      <c r="C20" s="19" t="n">
+      <c r="C21" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D20" s="20" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="15">
-      <c r="A21" s="21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="22" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="15">
+      <c r="A22" s="21" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
         <is>
           <t>OQ Group</t>
         </is>
       </c>
-      <c r="C21" s="23" t="n">
+      <c r="C22" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="D21" s="24" t="inlineStr">
+      <c r="D22" s="24" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="15">
-      <c r="A22" s="17" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="15">
+      <c r="A23" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>PDO</t>
         </is>
       </c>
-      <c r="C22" s="19" t="n">
+      <c r="C23" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="D22" s="20" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="15">
-      <c r="A23" s="21" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="22" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="15">
+      <c r="A24" s="21" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>Petrofac</t>
         </is>
       </c>
-      <c r="C23" s="23" t="n">
+      <c r="C24" s="23" t="n">
         <v>55</v>
       </c>
-      <c r="D23" s="24" t="inlineStr">
+      <c r="D24" s="24" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="15">
-      <c r="A24" s="17" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="15">
+      <c r="A25" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>Petronas</t>
         </is>
       </c>
-      <c r="C24" s="19" t="n">
+      <c r="C25" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="15">
-      <c r="A25" s="21" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="22" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="15">
+      <c r="A26" s="21" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
         <is>
           <t>QatarEnergy</t>
         </is>
       </c>
-      <c r="C25" s="23" t="n">
+      <c r="C26" s="23" t="n">
         <v>284</v>
       </c>
-      <c r="D25" s="24" t="inlineStr">
+      <c r="D26" s="24" t="inlineStr">
         <is>
           <t>2026-03-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="15">
-      <c r="A26" s="17" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
-        <is>
-          <t>QatarEnergy LNG</t>
-        </is>
-      </c>
-      <c r="C26" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="D26" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
         </is>
       </c>
     </row>
@@ -972,82 +967,82 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
+          <t>QatarEnergy LNG</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="15">
+      <c r="A28" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
           <t>Saipem</t>
         </is>
       </c>
-      <c r="C27" s="17" t="n">
+      <c r="C28" s="17" t="n">
         <v>195</v>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="15">
-      <c r="A28" s="21" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="22" t="inlineStr">
+    <row r="29" ht="15" customHeight="1" s="15">
+      <c r="A29" s="21" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
         <is>
           <t>Saudi Aramco</t>
         </is>
       </c>
-      <c r="C28" s="23" t="n">
+      <c r="C29" s="23" t="n">
         <v>221</v>
       </c>
-      <c r="D28" s="24" t="inlineStr">
+      <c r="D29" s="24" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="15">
-      <c r="A29" s="17" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="18" t="inlineStr">
+    <row r="30" ht="15" customHeight="1" s="15">
+      <c r="A30" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>Shell</t>
         </is>
       </c>
-      <c r="C29" s="19" t="n">
+      <c r="C30" s="19" t="n">
         <v>181</v>
       </c>
-      <c r="D29" s="20" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1" s="15">
-      <c r="A30" s="21" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="22" t="inlineStr">
+    <row r="31" ht="15" customHeight="1" s="15">
+      <c r="A31" s="21" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
         <is>
           <t>SLB</t>
         </is>
       </c>
-      <c r="C30" s="23" t="n">
+      <c r="C31" s="23" t="n">
         <v>824</v>
       </c>
-      <c r="D30" s="24" t="inlineStr">
+      <c r="D31" s="24" t="inlineStr">
         <is>
           <t>2026-03-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="15">
-      <c r="A31" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="18" t="inlineStr">
-        <is>
-          <t>Suncor</t>
-        </is>
-      </c>
-      <c r="C31" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D31" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -1057,61 +1052,79 @@
       </c>
       <c r="B32" s="18" t="inlineStr">
         <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="n">
+        <v>27</v>
+      </c>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
           <t>Technip Energies</t>
         </is>
       </c>
-      <c r="C32" s="17" t="n">
+      <c r="C33" s="17" t="n">
         <v>172</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="21" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="22" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="21" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
         <is>
           <t>TotalEnergies</t>
         </is>
       </c>
-      <c r="C33" s="23" t="n">
+      <c r="C34" s="23" t="n">
         <v>658</v>
       </c>
-      <c r="D33" s="24" t="inlineStr">
+      <c r="D34" s="24" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="17" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="18" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="17" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="18" t="inlineStr">
         <is>
           <t>Woodside Energy</t>
         </is>
       </c>
-      <c r="C34" s="19" t="n">
+      <c r="C35" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="D34" s="20" t="inlineStr">
+      <c r="D35" s="20" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="25" t="n"/>
-      <c r="B35" s="26" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="25" t="n"/>
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C35" s="27">
-        <f>SUM(C2:C34)</f>
+      <c r="C36" s="27">
+        <f>SUM(C2:C35)</f>
         <v/>
       </c>
-      <c r="D35" s="25" t="n"/>
+      <c r="D36" s="25" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Add Larsen & Toubro: 904 jobs across 9 countries
Scraped from PeopleStrong AltOne platform API.
Countries: India (784), Saudi Arabia (50), Oman (32), UAE (19),
Kuwait (6), Indonesia (6), Qatar (3), Uzbekistan (3), Guinea (1).
Total: 6,648 jobs | 35 companies | 130 countries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -792,21 +792,16 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="15">
-      <c r="A17" s="17" t="n">
+      <c r="A17" s="21" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>Mubadala Energy</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="D17" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>904</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="15">
@@ -815,29 +810,29 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
+          <t>Mubadala Energy</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="15">
+      <c r="A19" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
           <t>McDermott</t>
         </is>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C19" s="17" t="n">
         <v>357</v>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="15">
-      <c r="A19" s="21" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="22" t="inlineStr">
-        <is>
-          <t>NIOC</t>
-        </is>
-      </c>
-      <c r="C19" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="D19" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="15">
@@ -846,136 +841,136 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
+          <t>NIOC</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="15">
+      <c r="A21" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
           <t>NMDC</t>
         </is>
       </c>
-      <c r="C20" s="21" t="n">
+      <c r="C21" s="21" t="n">
         <v>52</v>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="15">
-      <c r="A21" s="17" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="15">
+      <c r="A22" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>North Oil Company</t>
         </is>
       </c>
-      <c r="C21" s="19" t="n">
+      <c r="C22" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D21" s="20" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="15">
-      <c r="A22" s="21" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="22" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="15">
+      <c r="A23" s="21" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>OQ Group</t>
         </is>
       </c>
-      <c r="C22" s="23" t="n">
+      <c r="C23" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="D23" s="24" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="15">
-      <c r="A23" s="17" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="15">
+      <c r="A24" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>PDO</t>
         </is>
       </c>
-      <c r="C23" s="19" t="n">
+      <c r="C24" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="D23" s="20" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="15">
-      <c r="A24" s="21" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="22" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="15">
+      <c r="A25" s="21" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
         <is>
           <t>Petrofac</t>
         </is>
       </c>
-      <c r="C24" s="23" t="n">
+      <c r="C25" s="23" t="n">
         <v>55</v>
       </c>
-      <c r="D24" s="24" t="inlineStr">
+      <c r="D25" s="24" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="15">
-      <c r="A25" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="15">
+      <c r="A26" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>Petronas</t>
         </is>
       </c>
-      <c r="C25" s="19" t="n">
+      <c r="C26" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="D25" s="20" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="15">
-      <c r="A26" s="21" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="22" t="inlineStr">
+    <row r="27" ht="15" customHeight="1" s="15">
+      <c r="A27" s="21" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
         <is>
           <t>QatarEnergy</t>
         </is>
       </c>
-      <c r="C26" s="23" t="n">
+      <c r="C27" s="23" t="n">
         <v>284</v>
       </c>
-      <c r="D26" s="24" t="inlineStr">
+      <c r="D27" s="24" t="inlineStr">
         <is>
           <t>2026-03-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="15">
-      <c r="A27" s="17" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="18" t="inlineStr">
-        <is>
-          <t>QatarEnergy LNG</t>
-        </is>
-      </c>
-      <c r="C27" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="D27" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
         </is>
       </c>
     </row>
@@ -985,82 +980,82 @@
       </c>
       <c r="B28" s="18" t="inlineStr">
         <is>
+          <t>QatarEnergy LNG</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="15">
+      <c r="A29" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
           <t>Saipem</t>
         </is>
       </c>
-      <c r="C28" s="17" t="n">
+      <c r="C29" s="17" t="n">
         <v>195</v>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="15">
-      <c r="A29" s="21" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="22" t="inlineStr">
+    <row r="30" ht="15" customHeight="1" s="15">
+      <c r="A30" s="21" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
         <is>
           <t>Saudi Aramco</t>
         </is>
       </c>
-      <c r="C29" s="23" t="n">
+      <c r="C30" s="23" t="n">
         <v>221</v>
       </c>
-      <c r="D29" s="24" t="inlineStr">
+      <c r="D30" s="24" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1" s="15">
-      <c r="A30" s="17" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="18" t="inlineStr">
+    <row r="31" ht="15" customHeight="1" s="15">
+      <c r="A31" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
         <is>
           <t>Shell</t>
         </is>
       </c>
-      <c r="C30" s="19" t="n">
+      <c r="C31" s="19" t="n">
         <v>181</v>
       </c>
-      <c r="D30" s="20" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="15">
-      <c r="A31" s="21" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="22" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="21" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
         <is>
           <t>SLB</t>
         </is>
       </c>
-      <c r="C31" s="23" t="n">
+      <c r="C32" s="23" t="n">
         <v>824</v>
       </c>
-      <c r="D31" s="24" t="inlineStr">
+      <c r="D32" s="24" t="inlineStr">
         <is>
           <t>2026-03-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="17" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="18" t="inlineStr">
-        <is>
-          <t>Suncor</t>
-        </is>
-      </c>
-      <c r="C32" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D32" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
         </is>
       </c>
     </row>
@@ -1070,61 +1065,79 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
+          <t>Suncor</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="n">
+        <v>27</v>
+      </c>
+      <c r="D33" s="20" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="18" t="inlineStr">
+        <is>
           <t>Technip Energies</t>
         </is>
       </c>
-      <c r="C33" s="17" t="n">
+      <c r="C34" s="17" t="n">
         <v>172</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="21" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="22" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="21" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="22" t="inlineStr">
         <is>
           <t>TotalEnergies</t>
         </is>
       </c>
-      <c r="C34" s="23" t="n">
+      <c r="C35" s="23" t="n">
         <v>658</v>
       </c>
-      <c r="D34" s="24" t="inlineStr">
+      <c r="D35" s="24" t="inlineStr">
         <is>
           <t>2026-03-06</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="17" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="18" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="18" t="inlineStr">
         <is>
           <t>Woodside Energy</t>
         </is>
       </c>
-      <c r="C35" s="19" t="n">
+      <c r="C36" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="25" t="n"/>
-      <c r="B36" s="26" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="25" t="n"/>
+      <c r="B37" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C36" s="27">
-        <f>SUM(C2:C35)</f>
+      <c r="C37" s="27">
+        <f>SUM(C2:C36)</f>
         <v/>
       </c>
-      <c r="D36" s="25" t="n"/>
+      <c r="D37" s="25" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Re-scrape SLB (843), Baker Hughes (742), TotalEnergies (658)
Updated job counts: SLB 824→843, Baker Hughes 741→742, TotalEnergies 658→658.
Total: 6,668 jobs | 35 companies | 126 countries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="C3" s="23" t="n">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="D3" s="24" t="inlineStr">
         <is>
@@ -1051,7 +1051,7 @@
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>824</v>
+        <v>843</v>
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Re-scrape ExxonMobil (536), Halliburton (522), BP (397)
Updated job data for entries #4-6. ExxonMobil 542→536, Halliburton 523→522,
BP 416→397. Updated SCRAPING_GUIDE.md with detailed methods — notably
Halliburton's old AJAX endpoint no longer works, replaced with HTML
pagination approach (?p=N, 15 jobs/page, parse a[data-job-id]).
Total: 6,642 jobs | 35 companies | 124 countries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="C5" s="23" t="n">
-        <v>416</v>
+        <v>397</v>
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="C11" s="19" t="n">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="C12" s="23" t="n">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Re-scrape companies #7-9: QatarEnergy (287), Saudi Aramco (221), Shell (175)
Updated job data for QatarEnergy, Saudi Aramco, and Shell. Updated scraping
guide with detailed Shell Workday API method. Rebuilt job board: 6,639 jobs
across 35 companies and 124 countries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -966,11 +966,11 @@
         </is>
       </c>
       <c r="C27" s="23" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
@@ -1033,11 +1033,11 @@
         </is>
       </c>
       <c r="C31" s="19" t="n">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="D31" s="20" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape BP via Workday API (393 jobs), update scraping guide
Switched BP scraping to Workday platform (bpinternational.wd3.myworkdayjobs.com)
as primary method. Previous Algolia Search method retained as backup.
TotalEnergies and ExxonMobil do not have Workday career sites.
Rebuilt job board: 6,635 jobs | 35 companies | 124 countries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -585,11 +585,11 @@
         </is>
       </c>
       <c r="C5" s="23" t="n">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape Petronas (29), Suncor (20), Mubadala Energy (40) — 6,627 total jobs
- Petronas: Oracle CX Recruiting, 29 jobs (all Malaysia)
- Suncor: Workday API, 20 jobs (17 Canada, 3 US)
- Mubadala Energy: careers-page.com SPA, 40 jobs (Indonesia, Malaysia, UAE)
- Updated SCRAPING_GUIDE.md with new methods and counts
- Updated Company_Tracker.xlsx

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -818,7 +818,7 @@
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -948,11 +948,11 @@
         </is>
       </c>
       <c r="C26" s="19" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -1069,11 +1069,11 @@
         </is>
       </c>
       <c r="C33" s="19" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D33" s="20" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add INPEX (73), Woodside Energy (15), ADNOC (67) job scrapes
Scraped companies #16-18 from the scraping guide:
- INPEX: 73 jobs (25 AU via SAP SuccessFactors + 48 ID via ASP.NET)
- Woodside Energy: 15 jobs from Taleo
- ADNOC: 67 jobs from Phenom People Vue.js SPA
Updated SCRAPING_GUIDE.md, Company_Tracker.xlsx, rebuilt job board (6,633 total jobs).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -531,11 +531,11 @@
         </is>
       </c>
       <c r="C2" s="19" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -747,11 +747,11 @@
         </is>
       </c>
       <c r="C14" s="23" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -1118,11 +1118,11 @@
         </is>
       </c>
       <c r="C36" s="19" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D36" s="20" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update CNOOC International (0), PDO (0), QatarEnergy LNG (17) job scrapes
Scraped companies #19-21 from the scraping guide:
- CNOOC International: 0 jobs (no current openings)
- PDO: 0 jobs (no current openings on PetroJobs.om)
- QatarEnergy LNG: 17 jobs from Taleo (up from 12)
Updated SCRAPING_GUIDE.md, Company_Tracker.xlsx, rebuilt job board (6,627 total jobs).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -639,11 +639,11 @@
         </is>
       </c>
       <c r="C8" s="23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -912,11 +912,11 @@
         </is>
       </c>
       <c r="C24" s="19" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -984,11 +984,11 @@
         </is>
       </c>
       <c r="C28" s="19" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update jobs for North Oil Company (#22), McDermott (#24), Saipem (#25)
- North Oil Company: 2 jobs (Qatar, Taleo)
- McDermott: 375 jobs across 19 countries (Oracle HCM API)
- Saipem: 202 jobs across 20 countries (NCorePlat JSON)
- Total: 6,652 jobs across 33 companies
- Updated SCRAPING_GUIDE.md, Company_Tracker.xlsx

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -832,7 +832,12 @@
         </is>
       </c>
       <c r="C19" s="17" t="n">
-        <v>357</v>
+        <v>375</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="15">
@@ -880,7 +885,7 @@
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1007,12 @@
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>195</v>
+        <v>202</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="15">

</xml_diff>

<commit_message>
Re-scrape #23 Dragon Oil (6), #26 Technip (171), #27 NMDC (68), #28 L&T (99)
Updated job data for 4 companies. Total: 5860 jobs, 33 companies.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -657,11 +657,11 @@
         </is>
       </c>
       <c r="C9" s="19" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,12 @@
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>904</v>
+        <v>99</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="15">
@@ -834,7 +839,7 @@
       <c r="C19" s="17" t="n">
         <v>375</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
@@ -868,7 +873,12 @@
         </is>
       </c>
       <c r="C21" s="21" t="n">
-        <v>52</v>
+        <v>68</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="15">
@@ -1009,7 +1019,7 @@
       <c r="C29" s="17" t="n">
         <v>202</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
@@ -1097,7 +1107,12 @@
         </is>
       </c>
       <c r="C34" s="17" t="n">
-        <v>172</v>
+        <v>171</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
Re-scrape L&T with full pagination: 928 jobs (was 99 due to missing totalRecords key)
Fixed API pagination bug - used totalRecords instead of count. Total: 6689 jobs.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -801,9 +801,9 @@
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>99</v>
-      </c>
-      <c r="D17" t="inlineStr">
+        <v>928</v>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
@@ -875,7 +875,7 @@
       <c r="C21" s="21" t="n">
         <v>68</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
@@ -1109,7 +1109,7 @@
       <c r="C34" s="17" t="n">
         <v>171</v>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="14" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>

</xml_diff>

<commit_message>
Re-scrape ENOC: 8 → 3 jobs, update guide and tracker
- Updated ENOC_Jobs.csv with 3 current jobs (was 8)
- Added ENOC section (#29) to SCRAPING_GUIDE.md with platform details
- Updated Company_Tracker.xlsx row 10
- Rebuilt job board: 6,684 jobs, 33 companies, 122 countries

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -675,11 +675,11 @@
         </is>
       </c>
       <c r="C10" s="23" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape OQ Group: 5 → 16 jobs, update guide and tracker
- Updated OQ_Group_Jobs.csv with 16 current jobs (was 5)
- Added OQ Group section (#30) to SCRAPING_GUIDE.md with platform details
- Updated Company_Tracker.xlsx row 23
- Rebuilt job board: 6,695 jobs, 33 companies, 122 countries

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -909,11 +909,11 @@
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -1164,6 +1164,9 @@
       </c>
       <c r="D37" s="25" t="n"/>
     </row>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <autoFilter ref="A1:D30"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Re-scrape KPC & KNPC: both have 0 active jobs, update guide and tracker
- KPC: No active campaigns on recruitment portal (was 5 placeholder jobs)
- KNPC: No careers page; recruits via KPC portal, also 0 campaigns
- Added KPC (#31) and KNPC (#32) sections to SCRAPING_GUIDE.md
- Updated Company_Tracker.xlsx rows 15-16
- Rebuilt job board: 6,685 jobs, 31 companies, 122 countries

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -765,11 +765,11 @@
         </is>
       </c>
       <c r="C15" s="19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D15" s="20" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
@@ -783,11 +783,11 @@
         </is>
       </c>
       <c r="C16" s="23" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add AECOM Energy business line: 361 jobs across 11 countries
- New company: AECOM (Energy business line only, filtered from 4,578 total)
- Created AECOM_Jobs.csv with 361 jobs (UK 144, US 131, India 30, Romania 13, Ireland 11, Australia 7, Poland 7, Spain 7, Canada 6, NZ 4, Philippines 1)
- Added AECOM section (#33) to SCRAPING_GUIDE.md with SmartRecruiters/Nuxt.js platform details
- Added AECOM to Company_Tracker.xlsx (row 37)
- Rebuilt job board: 7,046 jobs, 32 companies, 123 countries

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -1152,21 +1152,36 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="25" t="n"/>
-      <c r="B37" s="26" t="inlineStr">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>AECOM</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>361</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="25" t="n"/>
+      <c r="B38" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C37" s="27">
-        <f>SUM(C2:C36)</f>
+      <c r="C38" s="27">
+        <f>SUM(C2:C37)</f>
         <v/>
       </c>
-      <c r="D37" s="25" t="n"/>
-    </row>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
+      <c r="D38" s="25" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Update scraping guide and tracker with Repsol (51 jobs)
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="49">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -164,6 +164,9 @@
   </si>
   <si>
     <t xml:space="preserve">ENI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repsol</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -647,7 +650,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -1090,7 +1093,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="n">
         <v>31</v>
       </c>
@@ -1104,7 +1107,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="n">
         <v>32</v>
       </c>
@@ -1118,7 +1121,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="n">
         <v>33</v>
       </c>
@@ -1132,7 +1135,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="n">
         <v>34</v>
       </c>
@@ -1146,7 +1149,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="n">
         <v>35</v>
       </c>
@@ -1160,7 +1163,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="n">
         <v>36</v>
       </c>
@@ -1174,7 +1177,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="n">
         <v>37</v>
       </c>
@@ -1188,16 +1191,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11"/>
-      <c r="B39" s="12" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C39" s="13" t="n">
-        <f aca="false">SUM(C2:C38)</f>
-        <v>7126</v>
-      </c>
-      <c r="D39" s="11"/>
+      <c r="C39" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="11"/>
+      <c r="B40" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C40" s="13" t="n">
+        <f aca="false">SUM(C2:C39)</f>
+        <v>7177</v>
+      </c>
+      <c r="D40" s="11"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Update scraping guide and tracker with Sasol (72 jobs)
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="50">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -167,6 +167,9 @@
   </si>
   <si>
     <t xml:space="preserve">Repsol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sasol</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -650,7 +653,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -1205,16 +1208,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11"/>
-      <c r="B40" s="12" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C40" s="13" t="n">
-        <f aca="false">SUM(C2:C39)</f>
-        <v>7177</v>
-      </c>
-      <c r="D40" s="11"/>
+      <c r="C40" s="1" t="n">
+        <v>72</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="11"/>
+      <c r="B41" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C41" s="13" t="n">
+        <f aca="false">SUM(C2:C40)</f>
+        <v>7249</v>
+      </c>
+      <c r="D41" s="11"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Update scraping guide and tracker with Occidental (24 jobs)
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="51">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -170,6 +170,9 @@
   </si>
   <si>
     <t xml:space="preserve">Sasol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Occidental</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -653,7 +656,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -1222,16 +1225,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11"/>
-      <c r="B41" s="12" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C41" s="13" t="n">
-        <f aca="false">SUM(C2:C40)</f>
-        <v>7249</v>
-      </c>
-      <c r="D41" s="11"/>
+      <c r="C41" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="11"/>
+      <c r="B42" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C42" s="13" t="n">
+        <f aca="false">SUM(C2:C41)</f>
+        <v>7273</v>
+      </c>
+      <c r="D42" s="11"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Update scraping guide and tracker with EOG Resources (65 jobs)
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="52">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -173,6 +173,9 @@
   </si>
   <si>
     <t xml:space="preserve">Occidental</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EOG Resources</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -656,7 +659,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -1239,16 +1242,30 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="11"/>
-      <c r="B42" s="12" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C42" s="13" t="n">
-        <f aca="false">SUM(C2:C41)</f>
-        <v>7273</v>
-      </c>
-      <c r="D42" s="11"/>
+      <c r="C42" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="11"/>
+      <c r="B43" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C43" s="13" t="n">
+        <f aca="false">SUM(C2:C42)</f>
+        <v>7338</v>
+      </c>
+      <c r="D43" s="11"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Re-scrape SLB, Baker Hughes, TotalEnergies, ExxonMobil with fresh data
- SLB: 843 → 862 jobs (Coveo API, 81 countries)
- Baker Hughes: 742 → 761 jobs (Phenom HTML parsing, 58 countries)
- TotalEnergies: 658 → 670 jobs (custom portal HTML parsing, 54 countries)
- ExxonMobil: 536 → 521 jobs (SuccessFactors HTML parsing, 17 countries)
- Updated job board: 7,372 jobs, 35 companies, 123 countries
- Updated SCRAPING_GUIDE.md job counts and Company_Tracker.xlsx

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="C3" s="23" t="n">
-        <v>742</v>
+        <v>761</v>
       </c>
       <c r="D3" s="24" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C11" s="19" t="n">
-        <v>536</v>
+        <v>521</v>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>843</v>
+        <v>862</v>
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="C35" s="23" t="n">
-        <v>658</v>
+        <v>670</v>
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Re-scrape companies #9-#12: Shell (178), Chevron (199), Petrofac (55), ConocoPhillips (38)
Updated job board to 7435 jobs, 35 companies, 123 countries.
Updated scraping guide with detailed methods and working JS code for all 4 companies.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -64,7 +64,7 @@
     <t xml:space="preserve">Chevron</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-07</t>
+    <t xml:space="preserve">2026-03-12</t>
   </si>
   <si>
     <t xml:space="preserve">ConocoPhillips</t>
@@ -746,7 +746,7 @@
         <v>12</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>179</v>
+        <v>199</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>13</v>
@@ -760,7 +760,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>13</v>
@@ -1015,7 +1015,7 @@
         <v>55</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1096,10 +1096,10 @@
         <v>39</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C43" s="13" t="n">
         <f aca="false">SUM(C2:C42)</f>
-        <v>7404</v>
+        <v>7435</v>
       </c>
       <c r="D43" s="11"/>
     </row>

</xml_diff>

<commit_message>
Re-scrape companies #17-#20: Woodside (15), ADNOC (56), CNOOC (0), PDO (0)
Updated job board to 7425 jobs across 35 companies and 123 countries.
ADNOC decreased from 67 to 56 jobs. CNOOC and PDO remain at 0 jobs.
Updated SCRAPING_GUIDE.md with working extraction methods.
Updated Company_Tracker.xlsx with latest counts and dates.
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -539,11 +539,11 @@
         </is>
       </c>
       <c r="C2" s="19" t="n">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="D36" s="20" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Santos: 7 jobs scraped from recruitment.santos.com
New company #42. 7 jobs across 2 countries (Australia 5, Papua New Guinea 2).
Job board: 7432 jobs, 36 companies, 117 countries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -1268,17 +1268,29 @@
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="15">
-      <c r="A43" s="25" t="n"/>
+      <c r="A43" s="25" t="n">
+        <v>42</v>
+      </c>
       <c r="B43" s="26" t="inlineStr">
         <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="C43" s="27" t="n">
+        <v>7</v>
+      </c>
+      <c r="D43" s="25" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C43" s="27">
-        <f>SUM(C2:C42)</f>
+      <c r="C44">
+        <f>SUM(C2:C43)</f>
         <v/>
       </c>
-      <c r="D43" s="25" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>

</xml_diff>

<commit_message>
Add CNRL: 27 jobs scraped from 3 Oracle HCM career sites
Professional (17), New Graduate (1), Campus (9). All Canada.
Job board: 7459 jobs, 37 companies, 117 countries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -1282,13 +1282,26 @@
       <c r="D43" s="25" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" t="inlineStr">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>CNRL</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C44">
-        <f>SUM(C2:C43)</f>
+      <c r="C45">
+        <f>SUM(C2:C44)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Cenovus Energy: 42 jobs from Workday + contract portal
Workday (32 jobs) + Client Connections portal (10 contract jobs).
Countries: Canada 25, USA 17.
Job board: 7501 jobs, 38 companies, 117 countries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -1282,7 +1282,7 @@
       <c r="D43" s="25" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="14" t="n">
         <v>43</v>
       </c>
       <c r="B44" s="14" t="inlineStr">
@@ -1295,13 +1295,26 @@
       </c>
     </row>
     <row r="45">
-      <c r="B45" t="inlineStr">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Cenovus Energy</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C45">
-        <f>SUM(C2:C44)</f>
+      <c r="C46">
+        <f>SUM(C2:C45)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Marathon Petroleum: 117 jobs scraped from Workday
All USA. Top categories: Internship (30), Operations (22), Maintenance (16), Engineering (13).
Job board: 7618 jobs, 39 companies, 117 countries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="14" min="1" max="1"/>
@@ -1295,7 +1295,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="14" t="n">
         <v>44</v>
       </c>
       <c r="B45" s="14" t="inlineStr">
@@ -1308,13 +1308,26 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" t="inlineStr">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>Marathon Petroleum</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="n">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C46">
-        <f>SUM(C2:C45)</f>
+      <c r="C47">
+        <f>SUM(C2:C46)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Company_Tracker: BP 399, QatarEnergy 280, Saudi Aramco 227, Shell 177, Chevron 199 (2026-03-18)
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="54">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t xml:space="preserve">BP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-09</t>
   </si>
   <si>
     <t xml:space="preserve">Chevron</t>
@@ -741,10 +738,10 @@
         <v>10</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -752,13 +749,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>199</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -766,7 +763,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>38</v>
@@ -780,7 +777,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>0</v>
@@ -794,13 +791,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>6</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -808,13 +805,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -822,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>525</v>
@@ -836,7 +833,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>560</v>
@@ -850,7 +847,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>0</v>
@@ -864,7 +861,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>73</v>
@@ -878,13 +875,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -892,13 +889,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -906,13 +903,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C17" s="9" t="n">
         <v>928</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -920,7 +917,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" s="5" t="n">
         <v>40</v>
@@ -934,13 +931,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>375</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -948,7 +945,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>0</v>
@@ -962,13 +959,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>68</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -976,13 +973,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C22" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -990,13 +987,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>16</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1004,7 +1001,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>0</v>
@@ -1018,7 +1015,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C25" s="9" t="n">
         <v>55</v>
@@ -1032,7 +1029,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>29</v>
@@ -1046,13 +1043,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C27" s="9" t="n">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1060,13 +1057,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>17</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1074,13 +1071,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>202</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1088,13 +1085,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C30" s="9" t="n">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1102,13 +1099,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1116,7 +1113,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C32" s="9" t="n">
         <v>813</v>
@@ -1130,7 +1127,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>21</v>
@@ -1144,13 +1141,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>171</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1158,7 +1155,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C35" s="9" t="n">
         <v>686</v>
@@ -1172,7 +1169,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C36" s="5" t="n">
         <v>15</v>
@@ -1186,13 +1183,13 @@
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C37" s="1" t="n">
         <v>361</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1200,13 +1197,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C38" s="1" t="n">
         <v>80</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1214,13 +1211,13 @@
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C39" s="1" t="n">
         <v>51</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1228,13 +1225,13 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C40" s="1" t="n">
         <v>72</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1242,13 +1239,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C41" s="1" t="n">
         <v>24</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1256,13 +1253,13 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C42" s="1" t="n">
         <v>65</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1270,53 +1267,53 @@
         <v>42</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>7</v>
       </c>
       <c r="D43" s="11"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="n">
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C44" s="1" t="n">
         <v>27</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="n">
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C45" s="1" t="n">
         <v>42</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="n">
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C46" s="1" t="n">
         <v>117</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C47" s="1" t="n">
         <f aca="false">SUM(C2:C46)</f>
-        <v>7589</v>
+        <v>7576</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Company_Tracker: Petrofac 73, ConocoPhillips 39, Petronas 28, Suncor 23, Mubadala Energy 40
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -766,10 +766,10 @@
         <v>12</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -923,7 +923,7 @@
         <v>40</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1018,10 +1018,10 @@
         <v>31</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1032,10 +1032,10 @@
         <v>32</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1130,10 +1130,10 @@
         <v>39</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="C47" s="1" t="n">
         <f aca="false">SUM(C2:C46)</f>
-        <v>7576</v>
+        <v>7596</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Company_Tracker.xlsx: INPEX=73, ADNOC=54, Woodside=9, CNOOC=3, PDO=0 (total 7591)
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="53">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -40,13 +40,10 @@
     <t xml:space="preserve">ADNOC</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-12</t>
+    <t xml:space="preserve">2026-03-18</t>
   </si>
   <si>
     <t xml:space="preserve">Baker Hughes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-18</t>
   </si>
   <si>
     <t xml:space="preserve">Bapco Energies</t>
@@ -696,7 +693,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="5" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>5</v>
@@ -713,7 +710,7 @@
         <v>738</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -721,13 +718,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>11</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -735,13 +732,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>399</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -749,13 +746,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>199</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -763,13 +760,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>39</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -777,10 +774,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>5</v>
@@ -791,13 +788,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>6</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -805,13 +802,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -819,13 +816,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>525</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -833,13 +830,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>560</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -847,13 +844,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -861,7 +858,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>73</v>
@@ -875,13 +872,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -889,13 +886,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -903,13 +900,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C17" s="9" t="n">
         <v>928</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -917,13 +914,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C18" s="5" t="n">
         <v>40</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -931,13 +928,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>375</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -945,13 +942,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -959,13 +956,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>68</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -973,13 +970,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C22" s="5" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -987,13 +984,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>16</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1001,7 +998,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>0</v>
@@ -1015,13 +1012,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C25" s="9" t="n">
         <v>73</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1029,13 +1026,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>28</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1043,13 +1040,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C27" s="9" t="n">
         <v>280</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1057,13 +1054,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>17</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1071,13 +1068,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>202</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1085,13 +1082,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C30" s="9" t="n">
         <v>227</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1099,13 +1096,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>177</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1113,13 +1110,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C32" s="9" t="n">
         <v>813</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1127,13 +1124,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>23</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1141,13 +1138,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>171</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1155,13 +1152,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C35" s="9" t="n">
         <v>686</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1169,10 +1166,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>5</v>
@@ -1183,13 +1180,13 @@
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C37" s="1" t="n">
         <v>361</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1197,13 +1194,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C38" s="1" t="n">
         <v>80</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1211,13 +1208,13 @@
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C39" s="1" t="n">
         <v>51</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1225,13 +1222,13 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C40" s="1" t="n">
         <v>72</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1239,13 +1236,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C41" s="1" t="n">
         <v>24</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1253,13 +1250,13 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C42" s="1" t="n">
         <v>65</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1267,7 +1264,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>7</v>
@@ -1279,7 +1276,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C44" s="1" t="n">
         <v>27</v>
@@ -1290,7 +1287,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C45" s="1" t="n">
         <v>42</v>
@@ -1301,7 +1298,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C46" s="1" t="n">
         <v>117</v>
@@ -1309,11 +1306,11 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C47" s="1" t="n">
         <f aca="false">SUM(C2:C46)</f>
-        <v>7596</v>
+        <v>7591</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Company_Tracker.xlsx with #26-30 job counts (2026-03-19)
Technip Energies: 162 | NMDC: 71 | L&T: 955 | ENOC: 3 | OQ Group: 18

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -687,7 +687,7 @@
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -809,11 +809,11 @@
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>928</v>
+        <v>955</v>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -881,11 +881,11 @@
         </is>
       </c>
       <c r="C21" s="21" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -917,11 +917,11 @@
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -1115,11 +1115,11 @@
         </is>
       </c>
       <c r="C34" s="17" t="n">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Company_Tracker: AECOM=346, ENI=87, Repsol=55 (2026-03-19)
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -777,7 +777,7 @@
       </c>
       <c r="D15" s="20" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -1169,11 +1169,11 @@
         </is>
       </c>
       <c r="C37" s="14" t="n">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -1187,11 +1187,11 @@
         </is>
       </c>
       <c r="C38" s="14" t="n">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -1205,11 +1205,11 @@
         </is>
       </c>
       <c r="C39" s="14" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Company_Tracker: Sasol=64, Occidental=23, EOG=61, Bapco=10, NIOC=0 (2026-03-19)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -575,11 +575,11 @@
         </is>
       </c>
       <c r="C4" s="19" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="D20" s="24" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -1223,11 +1223,11 @@
         </is>
       </c>
       <c r="C40" s="14" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -1241,11 +1241,11 @@
         </is>
       </c>
       <c r="C41" s="14" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -1259,11 +1259,11 @@
         </is>
       </c>
       <c r="C42" s="14" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape companies #41-45: Santos, CNRL, Cenovus, Marathon (2026-03-19)
Updated job counts:
- Santos: 7 → 6 (-1)
- CNRL: 27 → 15 (-12)
- Cenovus Energy: 42 → 38 (-4)
- Marathon Petroleum: 117 → 107 (-10)
- INOC: 0 (unchanged, CAPTCHA blocked)

Total board: 7,572 jobs | 40 companies | 122 countries

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -741,7 +741,7 @@
       </c>
       <c r="D13" s="20" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
@@ -1277,9 +1277,13 @@
         </is>
       </c>
       <c r="C43" s="27" t="n">
-        <v>7</v>
-      </c>
-      <c r="D43" s="25" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="D43" s="25" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="15">
       <c r="A44" s="14" t="n">
@@ -1291,7 +1295,12 @@
         </is>
       </c>
       <c r="C44" s="14" t="n">
-        <v>27</v>
+        <v>15</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="15">
@@ -1304,7 +1313,12 @@
         </is>
       </c>
       <c r="C45" s="14" t="n">
-        <v>42</v>
+        <v>38</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="15">
@@ -1317,7 +1331,12 @@
         </is>
       </c>
       <c r="C46" s="14" t="n">
-        <v>117</v>
+        <v>107</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="15">

</xml_diff>

<commit_message>
Update Company_Tracker.xlsx with fresh scrape counts (2026-03-21)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -557,11 +557,11 @@
         </is>
       </c>
       <c r="C3" s="23" t="n">
-        <v>738</v>
+        <v>807</v>
       </c>
       <c r="D3" s="24" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -593,11 +593,11 @@
         </is>
       </c>
       <c r="C5" s="23" t="n">
-        <v>399</v>
+        <v>390</v>
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -611,11 +611,11 @@
         </is>
       </c>
       <c r="C6" s="19" t="n">
-        <v>199</v>
+        <v>171</v>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -701,11 +701,11 @@
         </is>
       </c>
       <c r="C11" s="19" t="n">
-        <v>525</v>
+        <v>516</v>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -719,11 +719,11 @@
         </is>
       </c>
       <c r="C12" s="23" t="n">
-        <v>560</v>
+        <v>567</v>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -1061,11 +1061,11 @@
         </is>
       </c>
       <c r="C31" s="19" t="n">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D31" s="20" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -1079,11 +1079,11 @@
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>813</v>
+        <v>829</v>
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -1133,11 +1133,11 @@
         </is>
       </c>
       <c r="C35" s="23" t="n">
-        <v>686</v>
+        <v>738</v>
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
       <c r="C44" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1315,7 +1315,7 @@
       <c r="C45" s="14" t="n">
         <v>38</v>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
@@ -1333,7 +1333,7 @@
       <c r="C46" s="14" t="n">
         <v>107</v>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>

</xml_diff>

<commit_message>
Update Company_Tracker.xlsx with job counts from 2026-03-21 scrape
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -18,8 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -120,7 +121,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -201,6 +202,12 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -539,12 +546,10 @@
         </is>
       </c>
       <c r="C2" s="19" t="n">
-        <v>54</v>
-      </c>
-      <c r="D2" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+        <v>31</v>
+      </c>
+      <c r="D2" s="28" t="n">
+        <v>46102</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="15">
@@ -629,12 +634,10 @@
         </is>
       </c>
       <c r="C7" s="23" t="n">
-        <v>39</v>
-      </c>
-      <c r="D7" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+        <v>40</v>
+      </c>
+      <c r="D7" s="29" t="n">
+        <v>46102</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="15">
@@ -647,12 +650,10 @@
         </is>
       </c>
       <c r="C8" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>46102</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="15">
@@ -755,12 +756,10 @@
         </is>
       </c>
       <c r="C14" s="23" t="n">
-        <v>73</v>
-      </c>
-      <c r="D14" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+        <v>23</v>
+      </c>
+      <c r="D14" s="29" t="n">
+        <v>46102</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="15">
@@ -829,10 +828,8 @@
       <c r="C18" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+      <c r="D18" s="28" t="n">
+        <v>46102</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="15">
@@ -937,10 +934,8 @@
       <c r="C24" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+      <c r="D24" s="28" t="n">
+        <v>46102</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="15">
@@ -953,12 +948,10 @@
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>73</v>
-      </c>
-      <c r="D25" s="24" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+        <v>63</v>
+      </c>
+      <c r="D25" s="29" t="n">
+        <v>46102</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="15">
@@ -971,12 +964,10 @@
         </is>
       </c>
       <c r="C26" s="19" t="n">
-        <v>28</v>
-      </c>
-      <c r="D26" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="D26" s="28" t="n">
+        <v>46102</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="15">
@@ -1097,12 +1088,10 @@
         </is>
       </c>
       <c r="C33" s="19" t="n">
-        <v>23</v>
-      </c>
-      <c r="D33" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="D33" s="28" t="n">
+        <v>46102</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="15">
@@ -1151,12 +1140,10 @@
         </is>
       </c>
       <c r="C36" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="D36" s="20" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
+        <v>6</v>
+      </c>
+      <c r="D36" s="28" t="n">
+        <v>46102</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="15">

</xml_diff>

<commit_message>
Update Company_Tracker.xlsx for #21-30 (March 2026)
Updated job counts and dates for 10 companies:
- QatarEnergy LNG: 14 | North Oil Company: 1 | Dragon Oil: 5
- McDermott: 381 | Saipem: 218 | Technip Energies: 166
- NMDC: 65 | Larsen & Toubro: 971 | ENOC: 2 | OQ Group: 13

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -666,11 +666,11 @@
         </is>
       </c>
       <c r="C9" s="19" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -684,11 +684,11 @@
         </is>
       </c>
       <c r="C10" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -808,11 +808,11 @@
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>955</v>
+        <v>971</v>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -842,11 +842,11 @@
         </is>
       </c>
       <c r="C19" s="17" t="n">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -878,11 +878,11 @@
         </is>
       </c>
       <c r="C21" s="21" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -914,11 +914,11 @@
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -1016,11 +1016,11 @@
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D29" s="14" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
@@ -1104,11 +1104,11 @@
         </is>
       </c>
       <c r="C34" s="17" t="n">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update job board: 7,392 jobs across 41 companies (2026-03-27)
- Re-scraped BP (387), Shell (186), Saudi Aramco (227), Petronas (30), PDO (5)
- Added INPEX Australia (24) + INPEX Indonesia (47), replacing old Inpex_Jobs.csv
- Updated Baker Hughes (720), ADNOC (40), Woodside Energy (12)
- Rebuilt ME_Oil_Gas_Jobs.html and index.html via build_job_board.py
- Updated Company_Tracker.xlsx with new counts and date 2026-03-27

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="51">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -40,18 +40,15 @@
     <t xml:space="preserve">ADNOC</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-03-27</t>
+  </si>
+  <si>
     <t xml:space="preserve">Baker Hughes</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-21</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bapco Energies</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-22</t>
-  </si>
-  <si>
     <t xml:space="preserve">BP</t>
   </si>
   <si>
@@ -77,9 +74,6 @@
   </si>
   <si>
     <t xml:space="preserve">INOC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-19</t>
   </si>
   <si>
     <t xml:space="preserve">INPEX</t>
@@ -693,10 +687,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="5" t="n">
-        <v>31</v>
-      </c>
-      <c r="D2" s="6" t="n">
-        <v>46102</v>
+        <v>40</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -704,13 +698,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>807</v>
+        <v>720</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -724,7 +718,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -732,13 +726,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -746,13 +740,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>171</v>
+        <v>62</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -760,13 +754,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>40</v>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>46102</v>
+        <v>44</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -774,13 +768,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="D8" s="10" t="n">
-        <v>46102</v>
+      <c r="D8" s="10" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -788,13 +782,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>5</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -802,13 +796,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>2</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -816,13 +810,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -830,13 +824,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>567</v>
+        <v>593</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -844,13 +838,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -858,13 +852,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>46102</v>
+        <v>71</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -872,13 +866,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -886,13 +880,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -900,13 +894,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C17" s="9" t="n">
         <v>971</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -914,13 +908,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C18" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="D18" s="6" t="n">
-        <v>46102</v>
+      <c r="D18" s="6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -928,13 +922,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>381</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -942,13 +936,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -956,13 +950,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>65</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -970,13 +964,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C22" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -984,13 +978,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>13</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -998,13 +992,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>46102</v>
+        <v>5</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1012,13 +1006,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>63</v>
-      </c>
-      <c r="D25" s="10" t="n">
-        <v>46102</v>
+        <v>60</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1026,13 +1020,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="D26" s="6" t="n">
-        <v>46102</v>
+        <v>30</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1040,13 +1034,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C27" s="9" t="n">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1054,13 +1048,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>14</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1068,13 +1062,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>218</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1082,13 +1076,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C30" s="9" t="n">
         <v>227</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1096,13 +1090,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1110,13 +1104,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C32" s="9" t="n">
-        <v>829</v>
+        <v>789</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1124,13 +1118,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="D33" s="6" t="n">
-        <v>46102</v>
+        <v>22</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1138,13 +1132,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>166</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1152,13 +1146,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C35" s="9" t="n">
-        <v>738</v>
+        <v>760</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1166,13 +1160,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="D36" s="6" t="n">
-        <v>46102</v>
+        <v>12</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1180,13 +1174,13 @@
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C37" s="1" t="n">
         <v>346</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1194,13 +1188,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C38" s="1" t="n">
         <v>25</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1208,13 +1202,13 @@
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C39" s="1" t="n">
         <v>55</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1222,13 +1216,13 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C40" s="1" t="n">
         <v>25</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1236,13 +1230,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C41" s="1" t="n">
         <v>23</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1250,13 +1244,13 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C42" s="1" t="n">
         <v>62</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1264,13 +1258,13 @@
         <v>42</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>5</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1278,13 +1272,13 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C44" s="1" t="n">
         <v>19</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1292,13 +1286,13 @@
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C45" s="1" t="n">
         <v>38</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1306,22 +1300,22 @@
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C46" s="1" t="n">
         <v>107</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C47" s="1" t="n">
         <f aca="false">SUM(C2:C46)</f>
-        <v>7506</v>
+        <v>7392</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix TotalEnergies dates/locations; rescrape 769 jobs (2026-03-28)
Date Posted column was storing URLs instead of actual dates.
Re-scraped all 769 TotalEnergies jobs with correct DD-MM-YYYY → YYYY-MM-DD
dates and country names. Board now 7468 jobs across 40 companies.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -1133,11 +1133,11 @@
         </is>
       </c>
       <c r="C35" s="23" t="n">
-        <v>760</v>
+        <v>769</v>
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Halliburton: add posting dates for all 580 jobs
- Re-scraped all 39 listing pages (580 current jobs, up from 537)
- Fetched individual job detail pages in parallel batches of 20 to extract
  datePosted from JSON-LD structured data (format: YYYY-M-D)
- All 580 jobs now have Date Posted populated (previously all empty)
- Updated Company_Tracker.xlsx: 580 jobs, 2026-03-28
- Updated SCRAPING_GUIDE.md: notes date extraction method via JSON-LD
- Rebuilt ME_Oil_Gas_Jobs.html / index.html: 7474 jobs | 41 companies
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -833,10 +833,10 @@
         <v>16</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>593</v>
+        <v>580</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1329,13 +1329,13 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="1" t="s">
         <v>52</v>
       </c>
       <c r="C48" s="1" t="n">
         <f aca="false">SUM(C2:C47)</f>
-        <v>7487</v>
+        <v>7474</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix EOG Resources: add posting dates for all 80 jobs
- Re-scraped via POST to /process_jobsearch.asp (80 current jobs, up from 62)
- Extracted dates from page text ("Posted M/D/YYYY" pattern)
- All 80 jobs now have Date Posted populated (previously all empty)
- Updated Company_Tracker.xlsx: 80 jobs, 2026-03-28
- Rebuilt HTML: 7492 jobs | 41 companies | 130 countries
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -1253,10 +1253,10 @@
         <v>46</v>
       </c>
       <c r="C42" s="1" t="n">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="C48" s="1" t="n">
         <f aca="false">SUM(C2:C47)</f>
-        <v>7474</v>
+        <v>7492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Re-scrape companies #11-20: add 370 new jobs, rebuild HTML to 7716 total
Updated CSVs (2026-03-29):
- Petrofac: 64 jobs (UK, UAE, Malaysia, India, others)
- ConocoPhillips: 43 jobs (USA, Australia, Norway, UK, Canada)
- Petronas: 25 jobs (Malaysia)
- Suncor: 27 jobs (Canada, USA)
- Mubadala Energy: 41 jobs (Indonesia, Malaysia, UAE)
- INPEX Australia: 25 jobs (Australia)
- INPEX Indonesia: 47 jobs (Indonesia)
- Woodside Energy: 11 jobs (Mexico, Australia, USA, UK)
- ADNOC: 30 jobs (UAE)
- CNOOC International: 9 jobs (Canada, UK)
- PDO: 0 jobs (site requires login)

HTML rebuilt: 7716 jobs | 41 companies

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -539,11 +539,11 @@
         </is>
       </c>
       <c r="C2" s="19" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -629,11 +629,11 @@
         </is>
       </c>
       <c r="C7" s="23" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -647,11 +647,11 @@
         </is>
       </c>
       <c r="C8" s="23" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -755,11 +755,11 @@
         </is>
       </c>
       <c r="C14" s="23" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -827,11 +827,11 @@
         </is>
       </c>
       <c r="C18" s="19" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -935,11 +935,11 @@
         </is>
       </c>
       <c r="C24" s="19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -953,11 +953,11 @@
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D25" s="24" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -971,11 +971,11 @@
         </is>
       </c>
       <c r="C26" s="19" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1097,11 +1097,11 @@
         </is>
       </c>
       <c r="C33" s="19" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D33" s="20" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1151,11 +1151,11 @@
         </is>
       </c>
       <c r="C36" s="19" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D36" s="20" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape companies #21-30: add L&T, ENOC, OQ, update all; rebuild HTML to 7748 total
- Larsen & Toubro (#28): 1,006 jobs via PeopleStrong API (India, UAE, Saudi Arabia, Oman…)
- ENOC (#29): 4 jobs (Dubai, UAE)
- OQ Group (#30): 9 jobs (Muscat / Sohar / Duqm, Oman)
- Saipem (#21): updated to 223 jobs
- Technip Energies (#26): updated to 179 jobs
- NMDC (#27): updated to 106 jobs
- McDermott, Dragon Oil, QatarEnergy LNG: minor count adjustments
- HTML board rebuilt: 7,748 jobs | 42 companies
- Company_Tracker.xlsx updated with latest counts and dates

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -665,11 +665,11 @@
         </is>
       </c>
       <c r="C9" s="19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -683,11 +683,11 @@
         </is>
       </c>
       <c r="C10" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -809,11 +809,11 @@
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>1012</v>
+        <v>1006</v>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -845,11 +845,11 @@
         </is>
       </c>
       <c r="C19" s="17" t="n">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -881,11 +881,11 @@
         </is>
       </c>
       <c r="C21" s="21" t="n">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -917,11 +917,11 @@
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1025,11 +1025,11 @@
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="D29" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1115,11 +1115,11 @@
         </is>
       </c>
       <c r="C34" s="17" t="n">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape companies #31-50: update 13 CSVs, rebuild HTML to 7844 total
Companies re-scraped:
- AECOM: 329 jobs (Energy BL, UK/US/India/Romania/other)
- Sasol: 55 jobs (South Africa/Germany/Mozambique/USA)
- Occidental: 41 jobs (USA/Algeria)
- EOG Resources: 84 jobs (USA)
- Bapco Energies: 10 jobs (Bahrain)
- Santos: 5 jobs (Australia)
- CNRL: 22 jobs (Canada)
- Cenovus Energy: 28 jobs (Canada/USA)
- Marathon Petroleum: 80 jobs (USA)
- ENI: 98 jobs (Italy/Germany/Netherlands/other)
- Repsol: 57 jobs (Spain/USA/other)
- SATORP: 19 jobs (Saudi Arabia, kept from prior scrape)

HTML rebuilt: 7844 jobs across 42 companies and 133 countries

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -579,7 +579,7 @@
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1223,11 +1223,11 @@
         </is>
       </c>
       <c r="C40" s="14" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1259,11 +1259,11 @@
         </is>
       </c>
       <c r="C42" s="14" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="D43" s="25" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1295,11 +1295,11 @@
         </is>
       </c>
       <c r="C44" s="14" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1313,11 +1313,11 @@
         </is>
       </c>
       <c r="C45" s="14" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1331,11 +1331,11 @@
         </is>
       </c>
       <c r="C46" s="14" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape companies #1-10: fresh job data (2026-03-30)
- SLB: 901 jobs
- Baker Hughes: 723 jobs (new CSV)
- TotalEnergies: 768 jobs
- ExxonMobil: 499 jobs
- Halliburton: 592 jobs
- BP: 382 jobs
- QatarEnergy: 284 jobs
- Saudi Aramco: 228 jobs (new CSV)
- Shell: 186 jobs
- Chevron: 187 jobs
- Rebuilt HTML job board: 8,812 total jobs across 42 companies
- Updated Company_Tracker.xlsx with new counts

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -557,11 +557,11 @@
         </is>
       </c>
       <c r="C3" s="23" t="n">
-        <v>730</v>
+        <v>723</v>
       </c>
       <c r="D3" s="24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -593,11 +593,11 @@
         </is>
       </c>
       <c r="C5" s="23" t="n">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -611,11 +611,11 @@
         </is>
       </c>
       <c r="C6" s="19" t="n">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -701,11 +701,11 @@
         </is>
       </c>
       <c r="C11" s="19" t="n">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -719,11 +719,11 @@
         </is>
       </c>
       <c r="C12" s="23" t="n">
-        <v>575</v>
+        <v>592</v>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -989,11 +989,11 @@
         </is>
       </c>
       <c r="C27" s="23" t="n">
-        <v>273</v>
+        <v>284</v>
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -1043,11 +1043,11 @@
         </is>
       </c>
       <c r="C30" s="23" t="n">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -1061,11 +1061,11 @@
         </is>
       </c>
       <c r="C31" s="19" t="n">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D31" s="20" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -1079,11 +1079,11 @@
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>898</v>
+        <v>901</v>
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>
@@ -1133,11 +1133,11 @@
         </is>
       </c>
       <c r="C35" s="23" t="n">
-        <v>774</v>
+        <v>768</v>
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape ADNOC (#18): fix title extraction, update from 30 to 40 jobs; rebuild HTML to 8822 total
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -539,11 +539,11 @@
         </is>
       </c>
       <c r="C2" s="19" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-03-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape companies #21-30: fresh data Apr 1 2026
- QatarEnergy LNG: 11 jobs
- North Oil Company: 2 jobs
- Dragon Oil: 4 jobs
- Saipem: 224 jobs (refreshed)
- Larsen & Toubro: 1009 unique jobs (full re-scrape via API)
- ENOC: 6 jobs
- OQ Group: 12 jobs
- Removed duplicate Baker_Hughes/Saudi_Aramco CSVs
- Rebuilt HTML board: 7877 jobs, 42 companies
- Updated Company_Tracker.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="D3" s="24" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -683,11 +683,11 @@
         </is>
       </c>
       <c r="C10" s="23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -809,11 +809,11 @@
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>1006</v>
+        <v>1009</v>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -885,7 +885,7 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -899,11 +899,11 @@
         </is>
       </c>
       <c r="C22" s="19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -917,11 +917,11 @@
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1007,11 +1007,11 @@
         </is>
       </c>
       <c r="C28" s="19" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1025,11 +1025,11 @@
         </is>
       </c>
       <c r="C29" s="17" t="n">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D29" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="D31" s="20" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1137,7 @@
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh jobs batch #31-50: AECOM, ENI, CNRL, Bapco, Repsol, EOG, Santos, SATORP, Sasol, Occidental, Marathon, Cenovus
- Re-scraped 11 companies: 7,799 total jobs across 42 companies
- Added: Cenovus_Jobs.csv (18), renamed from Cenovus_Energy_Jobs.csv
- Updated counts: AECOM 269, ENI 96, CNRL 27, Repsol 50, Occidental 42,
  EOG 80, Santos 4, SATORP 15, Marathon 84, Bapco 10, Sasol 55
- Rebuilt ME_Oil_Gas_Jobs.html job board
- Updated Company_Tracker.xlsx with latest counts

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -1169,11 +1169,11 @@
         </is>
       </c>
       <c r="C37" s="14" t="n">
-        <v>329</v>
+        <v>269</v>
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1187,11 +1187,11 @@
         </is>
       </c>
       <c r="C38" s="14" t="n">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1205,11 +1205,11 @@
         </is>
       </c>
       <c r="C39" s="14" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1241,11 +1241,11 @@
         </is>
       </c>
       <c r="C41" s="14" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1259,11 +1259,11 @@
         </is>
       </c>
       <c r="C42" s="14" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1277,11 +1277,11 @@
         </is>
       </c>
       <c r="C43" s="27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D43" s="25" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1295,11 +1295,11 @@
         </is>
       </c>
       <c r="C44" s="14" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1313,11 +1313,11 @@
         </is>
       </c>
       <c r="C45" s="14" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1331,11 +1331,11 @@
         </is>
       </c>
       <c r="C46" s="14" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
@@ -1349,11 +1349,11 @@
         </is>
       </c>
       <c r="C47" s="14" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape top 10 companies: SLB, Baker Hughes, TotalEnergies, ExxonMobil, Halliburton, BP, QatarEnergy, Saudi Aramco, Shell, Chevron
- Updated job counts across all 10 companies
- Rebuilt ME_Oil_Gas_Jobs.html (7499 jobs, 42 companies, 114 countries)
- Updated Company_Tracker.xlsx with latest counts

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="C3" s="23" t="n">
-        <v>723</v>
+        <v>698</v>
       </c>
       <c r="D3" s="24" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="C5" s="23" t="n">
-        <v>382</v>
+        <v>361</v>
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
@@ -611,7 +611,7 @@
         </is>
       </c>
       <c r="C6" s="19" t="n">
-        <v>187</v>
+        <v>152</v>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C11" s="19" t="n">
-        <v>499</v>
+        <v>461</v>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
@@ -719,7 +719,7 @@
         </is>
       </c>
       <c r="C12" s="23" t="n">
-        <v>592</v>
+        <v>604</v>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="C27" s="23" t="n">
-        <v>284</v>
+        <v>233</v>
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="C31" s="19" t="n">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="D31" s="20" t="inlineStr">
         <is>
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>901</v>
+        <v>797</v>
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="C35" s="23" t="n">
-        <v>768</v>
+        <v>756</v>
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Refresh top-10 company CSVs + rebuild job board (7,588 jobs)
Re-scraped SLB, Baker Hughes, TotalEnergies, ExxonMobil, Halliburton,
BP, QatarEnergy, Saudi Aramco, Shell, Chevron. Rebuilt ME_Oil_Gas_Jobs.html
and updated Company_Tracker.xlsx with latest counts.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -557,11 +557,11 @@
         </is>
       </c>
       <c r="C3" s="23" t="n">
-        <v>698</v>
+        <v>769</v>
       </c>
       <c r="D3" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -593,11 +593,11 @@
         </is>
       </c>
       <c r="C5" s="23" t="n">
-        <v>361</v>
+        <v>383</v>
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -611,11 +611,11 @@
         </is>
       </c>
       <c r="C6" s="19" t="n">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -701,11 +701,11 @@
         </is>
       </c>
       <c r="C11" s="19" t="n">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -719,11 +719,11 @@
         </is>
       </c>
       <c r="C12" s="23" t="n">
-        <v>604</v>
+        <v>625</v>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="D13" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="D15" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="D20" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -885,7 +885,7 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
       </c>
       <c r="D25" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -975,7 +975,7 @@
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -989,11 +989,11 @@
         </is>
       </c>
       <c r="C27" s="23" t="n">
-        <v>233</v>
+        <v>213</v>
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="D29" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1043,11 +1043,11 @@
         </is>
       </c>
       <c r="C30" s="23" t="n">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1061,11 +1061,11 @@
         </is>
       </c>
       <c r="C31" s="19" t="n">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="D31" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1079,11 +1079,11 @@
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>797</v>
+        <v>750</v>
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="D33" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1133,11 +1133,11 @@
         </is>
       </c>
       <c r="C35" s="23" t="n">
-        <v>756</v>
+        <v>784</v>
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="D36" s="20" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1227,7 @@
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="D43" s="25" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape companies #11-20: fresh data Apr 2 2026
Updated CSVs: Petrofac (48), ConocoPhillips (41), Petronas (25),
Mubadala Energy (40), ADNOC (49). Rebuilt HTML (7,574 jobs total).
Updated Company_Tracker.xlsx with new counts.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="C2" s="19" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
         </is>
       </c>
       <c r="C7" s="23" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="C18" s="19" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="D25" s="24" t="inlineStr">
         <is>
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="C33" s="19" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D33" s="20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Re-scrape companies #21-30 complete: fresh data Apr 2 2026
Updated CSVs: QatarEnergy LNG (11), North Oil Company (3), Dragon Oil (4),
McDermott (411), Saipem (201), Technip Energies (182), NMDC (57),
Larsen & Toubro (1035), ENOC (5), OQ Group (11).
Rebuilt ME_Oil_Gas_Jobs.html (7,556 jobs, 42 companies).
Updated Company_Tracker.xlsx totals.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -900,7 +900,7 @@
         <v>20</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>1009</v>
+        <v>1035</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>5</v>
@@ -928,7 +928,7 @@
         <v>22</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>5</v>
@@ -1068,7 +1068,7 @@
         <v>32</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>5</v>
@@ -1138,7 +1138,7 @@
         <v>37</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>5</v>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="C48" s="1" t="n">
         <f aca="false">SUM(C2:C47)</f>
-        <v>7525</v>
+        <v>7556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Re-scrape companies #41-46: fresh data as of 2026-04-02
- INOC (#41): 0 jobs (CAPTCHA-blocked)
- Santos (#42): 4 jobs (PageUp People ATS)
- CNRL (#43): 23 jobs (Oracle HCM, 3 sites)
- Cenovus Energy (#44): 21 jobs (Workday wd3 + contract portal)
- Marathon Petroleum (#45): 84 jobs (Workday wd1)
- SATORP (#46): 15 jobs (SAP SuccessFactors)
- Updated Company_Tracker.xlsx and rebuilt ME_Oil_Gas_Jobs.html (7619 total jobs)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -1295,7 +1295,7 @@
         </is>
       </c>
       <c r="C44" s="14" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="C45" s="14" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Motiva (#48): 7 jobs via Workday, rebuild HTML to 7802 jobs/43 companies
- New: Motiva_Jobs.csv — 7 jobs, all USA (Houston TX & Port Arthur TX)
- ATS: Workday wd1 (motiva/MotivaCareers), single API call pattern
- SCRAPING_GUIDE.md: Added entry #48 with full API details and reuse notes
- Rebuilt ME_Oil_Gas_Jobs.html + index.html: 7802 jobs | 43 companies | 135 countries
- Company_Tracker.xlsx: Added Motiva row, corrected 18 stale job counts to match CSVs,
  TOTAL formula updated to =SUM(C2:C49) = 7802

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="55">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -40,18 +40,18 @@
     <t xml:space="preserve">ADNOC</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-04-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baker Hughes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bapco Energies</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-04-02</t>
   </si>
   <si>
-    <t xml:space="preserve">Baker Hughes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bapco Energies</t>
-  </si>
-  <si>
     <t xml:space="preserve">BP</t>
   </si>
   <si>
@@ -182,6 +182,9 @@
   </si>
   <si>
     <t xml:space="preserve">Sembcorp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motiva</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -310,7 +313,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -365,6 +368,10 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -665,7 +672,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -696,7 +703,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="5" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>5</v>
@@ -713,7 +720,7 @@
         <v>711</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -721,13 +728,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>10</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -741,7 +748,7 @@
         <v>390</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -755,7 +762,7 @@
         <v>179</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -769,7 +776,7 @@
         <v>37</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -780,7 +787,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>5</v>
@@ -794,7 +801,7 @@
         <v>13</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>5</v>
@@ -808,7 +815,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>5</v>
@@ -825,7 +832,7 @@
         <v>493</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -839,7 +846,7 @@
         <v>619</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -853,7 +860,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -864,7 +871,7 @@
         <v>18</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>5</v>
@@ -881,7 +888,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -895,7 +902,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -906,7 +913,7 @@
         <v>21</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>5</v>
@@ -923,7 +930,7 @@
         <v>37</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -934,7 +941,7 @@
         <v>23</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>5</v>
@@ -951,7 +958,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -962,7 +969,7 @@
         <v>25</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>5</v>
@@ -976,7 +983,7 @@
         <v>26</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>5</v>
@@ -990,7 +997,7 @@
         <v>27</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>5</v>
@@ -1007,7 +1014,7 @@
         <v>0</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1021,7 +1028,7 @@
         <v>46</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1035,7 +1042,7 @@
         <v>25</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1049,7 +1056,7 @@
         <v>232</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1060,7 +1067,7 @@
         <v>32</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>5</v>
@@ -1074,7 +1081,7 @@
         <v>33</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>5</v>
@@ -1091,7 +1098,7 @@
         <v>229</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1105,7 +1112,7 @@
         <v>179</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1119,7 +1126,7 @@
         <v>828</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1133,7 +1140,7 @@
         <v>25</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1144,7 +1151,7 @@
         <v>38</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>5</v>
@@ -1161,7 +1168,7 @@
         <v>803</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1172,7 +1179,7 @@
         <v>40</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>5</v>
@@ -1189,7 +1196,7 @@
         <v>310</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1200,7 +1207,7 @@
         <v>42</v>
       </c>
       <c r="C38" s="1" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>5</v>
@@ -1214,7 +1221,7 @@
         <v>43</v>
       </c>
       <c r="C39" s="1" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>5</v>
@@ -1231,7 +1238,7 @@
         <v>53</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1242,7 +1249,7 @@
         <v>45</v>
       </c>
       <c r="C41" s="1" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>5</v>
@@ -1259,7 +1266,7 @@
         <v>79</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1273,7 +1280,7 @@
         <v>4</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1287,7 +1294,7 @@
         <v>23</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1298,7 +1305,7 @@
         <v>49</v>
       </c>
       <c r="C45" s="1" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>5</v>
@@ -1315,7 +1322,7 @@
         <v>84</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1329,7 +1336,7 @@
         <v>15</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1343,16 +1350,30 @@
         <v>82</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="1" t="s">
+      <c r="A49" s="14" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C49" s="1" t="n">
-        <f aca="false">SUM(C2:C48)</f>
-        <v>7761</v>
+      <c r="C49" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C50" s="1" t="n">
+        <f aca="false">SUM(C2:C49)</f>
+        <v>7802</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Brunel (277 jobs) — now 8079 jobs across 44 companies
- Scraped 277 jobs from Brunel via internal Next.js API proxy
  (POST /api/search/PublicationsSearch/Get with countryPreset filter)
- Added SCRAPING_GUIDE.md entry #49 with full API details, pagination,
  country normalization, and link construction pattern
- Updated Company_Tracker.xlsx with Brunel row (49, 277 jobs, 2026-04-05)
- Rebuilt HTML job board: 8079 jobs | 44 companies | 136 countries

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="56">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -185,6 +185,9 @@
   </si>
   <si>
     <t xml:space="preserve">Motiva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brunel</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -672,7 +675,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -1367,13 +1370,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="1" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C50" s="1" t="n">
-        <f aca="false">SUM(C2:C49)</f>
-        <v>7802</v>
+      <c r="C50" s="14" t="n">
+        <v>277</v>
+      </c>
+      <c r="D50" s="14" t="n">
+        <v>46117</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C51" s="1" t="n">
+        <f aca="false">SUM(C2:C50)</f>
+        <v>8079</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add KBR (1340 jobs) — now 9419 jobs across 45 companies
- Scraped 1340 jobs from KBR via Workday wd5 API
  (kbr.wd5.myworkdayjobs.com/wday/cxs/kbr/KBR_Careers/jobs)
- Added SCRAPING_GUIDE.md entry #50 with full details: parallel
  batch fetching, country extraction, multi-location handling,
  and browser console export method for proxy-blocked domains
- Updated Company_Tracker.xlsx with KBR row (50, 1340 jobs, 2026-04-06)
- Rebuilt HTML job board: 9419 jobs | 45 companies | 144 countries
- Top KBR locations: USA (804), Australia (96), Saudi Arabia (68),
  Iraq (64), UAE (57), India (47), Diego Garcia/BIOT (46)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="57">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -188,6 +188,9 @@
   </si>
   <si>
     <t xml:space="preserve">Brunel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KBR</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -675,7 +678,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -1384,13 +1387,27 @@
         <v>46117</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="1" t="s">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C51" s="1" t="n">
-        <f aca="false">SUM(C2:C50)</f>
-        <v>8079</v>
+      <c r="C51" s="14" t="n">
+        <v>1340</v>
+      </c>
+      <c r="D51" s="14" t="n">
+        <v>46118</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C52" s="1" t="n">
+        <f aca="false">SUM(C2:C51)</f>
+        <v>9419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Fluor (752 jobs) — now 10171 jobs across 46 companies
- Scraped 752 jobs from Fluor via EightFold.ai jobs API
  (GET /api/apply/v2/jobs?domain=fluor.com&start=N&num=10)
- Added SCRAPING_GUIDE.md entry #51 with EightFold API details:
  pagination via start offset, Redux store for total count,
  Unix timestamp date conversion, browser console export method
- Updated Company_Tracker.xlsx with Fluor row (51, 752, 2026-04-06)
- Rebuilt HTML job board: 10171 jobs | 46 companies | 145 countries
- Top Fluor locations: USA (592), Canada (53), India (42),
  Philippines (16), Poland (8), South Africa (7)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="58">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -191,6 +191,9 @@
   </si>
   <si>
     <t xml:space="preserve">KBR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluor</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -678,7 +681,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -1401,13 +1404,27 @@
         <v>46118</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="1" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="C52" s="1" t="n">
-        <f aca="false">SUM(C2:C51)</f>
-        <v>9419</v>
+      <c r="C52" s="14" t="n">
+        <v>752</v>
+      </c>
+      <c r="D52" s="14" t="n">
+        <v>46118</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C53" s="1" t="n">
+        <f aca="false">SUM(C2:C52)</f>
+        <v>10171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Wood (958 jobs) — Oracle HCM; now 11,129 jobs across 47 companies
- Wood_Jobs.csv: 958 jobs from Oracle HCM Fusion Cloud REST API
- Top countries: USA (162), Colombia (119), Chile (110), Canada (82), UK (81), Thailand (68)
- SCRAPING_GUIDE.md: added entry #52 with Oracle HCM pagination pattern
- Company_Tracker.xlsx: row 52 Wood/958, SUM updated to C2:C53
- HTML job board: 11,129 jobs | 47 companies | 146 countries

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="60">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -194,6 +194,12 @@
   </si>
   <si>
     <t xml:space="preserve">Fluor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-05</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -681,7 +687,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -1418,15 +1424,31 @@
         <v>46118</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="n">
+        <v>52</v>
+      </c>
       <c r="B53" s="1" t="s">
         <v>57</v>
       </c>
       <c r="C53" s="1" t="n">
-        <f aca="false">SUM(C2:C52)</f>
-        <v>10171</v>
-      </c>
-    </row>
+        <v>958</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C54" s="1" t="n">
+        <f aca="false">SUM(C2:C53)</f>
+        <v>11129</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <autoFilter ref="A1:D30"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Add Worley (793 jobs) — EightFold PCSX; now 11,922 jobs across 48 companies
- Worley_Jobs.csv: 793 jobs via /api/pcsx/search (EightFold PCSX platform)
- Top countries: USA (189), Canada (114), India (105), Colombia (54), Argentina (50), UAE (34)
- SCRAPING_GUIDE.md: added entry #53 with PCSX search API and discovery notes
- Company_Tracker.xlsx: row 53 Worley/793, SUM updated to C2:C54
- HTML job board: 11,922 jobs | 48 companies | 147 countries

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="61">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -200,6 +200,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-04-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worley</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -687,7 +690,7 @@
     <tabColor rgb="FF2F5496"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -1438,17 +1441,29 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1" t="n">
+        <v>53</v>
+      </c>
       <c r="B54" s="1" t="s">
         <v>59</v>
       </c>
       <c r="C54" s="1" t="n">
-        <f aca="false">SUM(C2:C53)</f>
-        <v>11129</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>793</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B55" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C55" s="1" t="n">
+        <f aca="false">SUM(C2:C54)</f>
+        <v>11922</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D30"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Fix SLB_Jobs.csv: remove 8 corrupted SLBCHUNK rows, update to 901 clean jobs
- Removed 8 rows where chunk labels (SLBCHUNK_1-8) appeared as job titles
- Regenerated SLB_Jobs.csv from original SLB1/SLB2 raw data: 901 unique jobs
- Fixed 1 title with stray numeric prefix ('02215899Sales Engineer' → 'Sales Engineer')
- Company_Tracker.xlsx: updated SLB count 828 → 901
- HTML job board: 11,995 jobs | 48 companies | 140 countries

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="62">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t xml:space="preserve">SLB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-06</t>
   </si>
   <si>
     <t xml:space="preserve">Suncor</t>
@@ -1141,10 +1144,10 @@
         <v>36</v>
       </c>
       <c r="C32" s="9" t="n">
-        <v>828</v>
+        <v>901</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1152,7 +1155,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>25</v>
@@ -1166,7 +1169,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>193</v>
@@ -1180,7 +1183,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C35" s="9" t="n">
         <v>803</v>
@@ -1194,7 +1197,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C36" s="5" t="n">
         <v>8</v>
@@ -1208,7 +1211,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C37" s="1" t="n">
         <v>310</v>
@@ -1222,7 +1225,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C38" s="1" t="n">
         <v>98</v>
@@ -1236,7 +1239,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C39" s="1" t="n">
         <v>55</v>
@@ -1250,7 +1253,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C40" s="1" t="n">
         <v>53</v>
@@ -1264,7 +1267,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C41" s="1" t="n">
         <v>39</v>
@@ -1278,7 +1281,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C42" s="1" t="n">
         <v>79</v>
@@ -1292,7 +1295,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>4</v>
@@ -1306,7 +1309,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C44" s="1" t="n">
         <v>23</v>
@@ -1320,7 +1323,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C45" s="1" t="n">
         <v>39</v>
@@ -1334,7 +1337,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C46" s="1" t="n">
         <v>84</v>
@@ -1348,7 +1351,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C47" s="1" t="n">
         <v>15</v>
@@ -1362,7 +1365,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C48" s="1" t="n">
         <v>82</v>
@@ -1376,7 +1379,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C49" s="14" t="n">
         <v>7</v>
@@ -1390,7 +1393,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C50" s="14" t="n">
         <v>277</v>
@@ -1404,7 +1407,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C51" s="14" t="n">
         <v>1340</v>
@@ -1418,7 +1421,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C52" s="14" t="n">
         <v>752</v>
@@ -1432,13 +1435,13 @@
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C53" s="1" t="n">
         <v>958</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1446,22 +1449,22 @@
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C54" s="1" t="n">
         <v>793</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C55" s="1" t="n">
         <f aca="false">SUM(C2:C54)</f>
-        <v>11922</v>
+        <v>11995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Re-scrape #16-30: fresh data for 12 companies, 11,865 total jobs
Companies re-scraped with Apr 7 2026 data:
- INPEX (AU+ID): 44 jobs — SAP SF + ASP.NET postback pagination
- Woodside: 7 jobs — Taleo single page
- ADNOC: 47 jobs — Phenom People, 5-page localStorage scrape
- QatarEnergy LNG: 11 jobs — Taleo tr.data-row
- North Oil Company: 4 jobs — Taleo tr.data-row
- Dragon Oil: 4 jobs — SAP SuccessFactors
- McDermott: 396 jobs — Oracle HCM REST API
- Technip Energies: 190 jobs — Oracle HCM REST API (ISO country codes)
- NMDC: 87 jobs — Oracle HCM REST API
- Saipem: 200 jobs — positions_saipem.json static fetch
- Larsen & Toubro: 1,013 jobs — PeopleStrong REST API
- ENOC: 6 jobs — TalentBrew single page
- OQ Group: 11 jobs — Taleo tr.data-row

Housekeeping: replaced split INPEX_AU/INPEX_ID, Dragon_Oil, NorthOilCompany,
and Woodside_Energy CSVs with unified canonical filenames.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -545,11 +545,11 @@
         </is>
       </c>
       <c r="C2" s="20" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D2" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="D3" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -671,11 +671,11 @@
         </is>
       </c>
       <c r="C9" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -689,11 +689,11 @@
         </is>
       </c>
       <c r="C10" s="24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -761,11 +761,11 @@
         </is>
       </c>
       <c r="C14" s="24" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -815,11 +815,11 @@
         </is>
       </c>
       <c r="C17" s="24" t="n">
-        <v>1034</v>
+        <v>1013</v>
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -851,11 +851,11 @@
         </is>
       </c>
       <c r="C19" s="18" t="n">
-        <v>408</v>
+        <v>396</v>
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -887,11 +887,11 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="D22" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -923,11 +923,11 @@
         </is>
       </c>
       <c r="C23" s="24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D23" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -1013,11 +1013,11 @@
         </is>
       </c>
       <c r="C28" s="20" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D28" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -1031,11 +1031,11 @@
         </is>
       </c>
       <c r="C29" s="18" t="n">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -1121,11 +1121,11 @@
         </is>
       </c>
       <c r="C34" s="18" t="n">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
@@ -1157,11 +1157,11 @@
         </is>
       </c>
       <c r="C36" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D36" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape #31-45: fresh data for 8 companies, 11,882 total jobs
Companies updated with Apr 8 2026 data:
- AECOM: 310 → 325 jobs (Energy business line, SmartRecruiters)
- ENI: updated formatting and date parsing (98 jobs, Oracle HCM)
- Repsol: 55 → 59 jobs (Workday)
- Occidental: 39 → 40 jobs (Workday)
- Cenovus Energy: 39 → 28 jobs (Workday, refreshed)
- Marathon Petroleum: 84 → 92 jobs (Workday)
- ME_Oil_Gas_Jobs.html rebuilt: 11,882 jobs across 53 companies
- Company_Tracker.xlsx updated with latest counts and dates

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -1175,11 +1175,11 @@
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="D37" s="15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1211,11 +1211,11 @@
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1247,11 +1247,11 @@
         </is>
       </c>
       <c r="C41" s="15" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D41" s="15" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1319,11 +1319,11 @@
         </is>
       </c>
       <c r="C45" s="15" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1337,11 +1337,11 @@
         </is>
       </c>
       <c r="C46" s="15" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add jobs for companies #46-53 (SATORP, Sembcorp, Motiva, Brunel, KBR, Fluor, Wood, Worley)
Fresh CSVs: KBR(1350), Fluor(744), Wood(946), Worley(831), Brunel(277), SATORP(15), Sembcorp(81), Motiva(7)
Total: 11,909 jobs across 48 companies — rebuilt HTML job board + updated tracker

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -1359,7 +1359,7 @@
       </c>
       <c r="D47" s="15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1373,11 +1373,11 @@
         </is>
       </c>
       <c r="C48" s="15" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="D49" s="29" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="D50" s="29" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1427,11 +1427,11 @@
         </is>
       </c>
       <c r="C51" s="29" t="n">
-        <v>1340</v>
+        <v>1350</v>
       </c>
       <c r="D51" s="29" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1445,11 +1445,11 @@
         </is>
       </c>
       <c r="C52" s="29" t="n">
-        <v>752</v>
+        <v>744</v>
       </c>
       <c r="D52" s="29" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1463,11 +1463,11 @@
         </is>
       </c>
       <c r="C53" s="15" t="n">
-        <v>958</v>
+        <v>946</v>
       </c>
       <c r="D53" s="15" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
@@ -1481,11 +1481,11 @@
         </is>
       </c>
       <c r="C54" s="15" t="n">
-        <v>793</v>
+        <v>831</v>
       </c>
       <c r="D54" s="15" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape #1-20: fresh data for all 20 priority companies, 11,984 total jobs
Companies updated (20): SLB (832), Baker Hughes (732), TotalEnergies (823),
ExxonMobil (489), Halliburton (635), BP (388), QatarEnergy (232),
Saudi Aramco (234), Shell (181), Chevron (219), Petrofac (42),
ConocoPhillips (28), Petronas (29), Mubadala Energy (39), INPEX (45),
Woodside (8), ADNOC (40), CNOOC International (4), PDO (0).
Suncor (0) — Workday maintenance blocked scrape.
Renamed CNOOC_International_Jobs.csv → CNOOCInternational_Jobs.csv.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -545,11 +545,11 @@
         </is>
       </c>
       <c r="C2" s="20" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="D2" s="21" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -563,11 +563,11 @@
         </is>
       </c>
       <c r="C3" s="24" t="n">
-        <v>711</v>
+        <v>732</v>
       </c>
       <c r="D3" s="25" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -599,11 +599,11 @@
         </is>
       </c>
       <c r="C5" s="24" t="n">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="D5" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -617,11 +617,11 @@
         </is>
       </c>
       <c r="C6" s="20" t="n">
-        <v>179</v>
+        <v>219</v>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -635,11 +635,11 @@
         </is>
       </c>
       <c r="C7" s="24" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -653,11 +653,11 @@
         </is>
       </c>
       <c r="C8" s="24" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -707,11 +707,11 @@
         </is>
       </c>
       <c r="C11" s="20" t="n">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -725,11 +725,11 @@
         </is>
       </c>
       <c r="C12" s="24" t="n">
-        <v>612</v>
+        <v>635</v>
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -761,11 +761,11 @@
         </is>
       </c>
       <c r="C14" s="24" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -833,11 +833,11 @@
         </is>
       </c>
       <c r="C18" s="20" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D18" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -945,7 +945,7 @@
       </c>
       <c r="D24" s="21" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -959,11 +959,11 @@
         </is>
       </c>
       <c r="C25" s="24" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D25" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -977,11 +977,11 @@
         </is>
       </c>
       <c r="C26" s="20" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D26" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
       </c>
       <c r="D27" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1049,11 +1049,11 @@
         </is>
       </c>
       <c r="C30" s="24" t="n">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D30" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1067,11 +1067,11 @@
         </is>
       </c>
       <c r="C31" s="20" t="n">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D31" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1085,11 +1085,11 @@
         </is>
       </c>
       <c r="C32" s="24" t="n">
-        <v>821</v>
+        <v>832</v>
       </c>
       <c r="D32" s="25" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1103,11 +1103,11 @@
         </is>
       </c>
       <c r="C33" s="20" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="D33" s="21" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1139,11 +1139,11 @@
         </is>
       </c>
       <c r="C35" s="24" t="n">
-        <v>803</v>
+        <v>823</v>
       </c>
       <c r="D35" s="25" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1157,11 +1157,11 @@
         </is>
       </c>
       <c r="C36" s="20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D36" s="21" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-scrape companies #41-53 (2026-04-10)
Santos(5), CNRL(31), Cenovus(22), Marathon(116), SATORP(15),
Sembcorp(78), Motiva(11), Brunel(286), KBR(1352), Fluor(766),
Wood(941), Worley(818) — total 12,037 jobs across 47 companies.
Updated ME_Oil_Gas_Jobs.html and Company_Tracker.xlsx.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Company_Tracker.xlsx
+++ b/Company_Tracker.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="D4" s="21" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -671,11 +671,11 @@
         </is>
       </c>
       <c r="C9" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -689,11 +689,11 @@
         </is>
       </c>
       <c r="C10" s="24" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="D16" s="25" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -815,11 +815,11 @@
         </is>
       </c>
       <c r="C17" s="24" t="n">
-        <v>1013</v>
+        <v>1038</v>
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="D20" s="25" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -887,11 +887,11 @@
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="D22" s="21" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="D23" s="25" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1013,11 +1013,11 @@
         </is>
       </c>
       <c r="C28" s="20" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D28" s="21" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1031,11 +1031,11 @@
         </is>
       </c>
       <c r="C29" s="18" t="n">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1121,11 +1121,11 @@
         </is>
       </c>
       <c r="C34" s="18" t="n">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1175,11 +1175,11 @@
         </is>
       </c>
       <c r="C37" s="15" t="n">
-        <v>325</v>
+        <v>280</v>
       </c>
       <c r="D37" s="15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1193,11 +1193,11 @@
         </is>
       </c>
       <c r="C38" s="15" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D38" s="15" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1211,11 +1211,11 @@
         </is>
       </c>
       <c r="C39" s="15" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="D40" s="15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1247,11 +1247,11 @@
         </is>
       </c>
       <c r="C41" s="15" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D41" s="15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1265,11 +1265,11 @@
         </is>
       </c>
       <c r="C42" s="15" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D42" s="15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1283,11 +1283,11 @@
         </is>
       </c>
       <c r="C43" s="28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D43" s="26" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1301,11 +1301,11 @@
         </is>
       </c>
       <c r="C44" s="15" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1319,11 +1319,11 @@
         </is>
       </c>
       <c r="C45" s="15" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1337,11 +1337,11 @@
         </is>
       </c>
       <c r="C46" s="15" t="n">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="D47" s="15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1373,11 +1373,11 @@
         </is>
       </c>
       <c r="C48" s="15" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1391,11 +1391,11 @@
         </is>
       </c>
       <c r="C49" s="29" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D49" s="29" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1409,11 +1409,11 @@
         </is>
       </c>
       <c r="C50" s="29" t="n">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="D50" s="29" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1427,11 +1427,11 @@
         </is>
       </c>
       <c r="C51" s="29" t="n">
-        <v>1350</v>
+        <v>1352</v>
       </c>
       <c r="D51" s="29" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1445,11 +1445,11 @@
         </is>
       </c>
       <c r="C52" s="29" t="n">
-        <v>744</v>
+        <v>766</v>
       </c>
       <c r="D52" s="29" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1463,11 +1463,11 @@
         </is>
       </c>
       <c r="C53" s="15" t="n">
-        <v>946</v>
+        <v>941</v>
       </c>
       <c r="D53" s="15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1481,11 +1481,11 @@
         </is>
       </c>
       <c r="C54" s="15" t="n">
-        <v>831</v>
+        <v>818</v>
       </c>
       <c r="D54" s="15" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1498,6 +1498,11 @@
       <c r="C55" s="15">
         <f>SUM(C2:C54)</f>
         <v/>
+      </c>
+      <c r="D55" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>